<commit_message>
dados: 2026-10-24 08:20 (132 arquivos)
</commit_message>
<xml_diff>
--- a/xlsx/dre/DRE_03_2026.xlsx
+++ b/xlsx/dre/DRE_03_2026.xlsx
@@ -588,21 +588,6 @@
     <t>R$  4.689,29</t>
   </si>
   <si>
-    <t>12/1</t>
-  </si>
-  <si>
-    <t>MP Interiores e Serv Ltda</t>
-  </si>
-  <si>
-    <t>R$  736,71</t>
-  </si>
-  <si>
-    <t>23/04/26</t>
-  </si>
-  <si>
-    <t>Digisac</t>
-  </si>
-  <si>
     <t>5/1</t>
   </si>
   <si>
@@ -614,6 +599,21 @@
   <si>
     <t xml:space="preserve">Reembolso Pushing
 </t>
+  </si>
+  <si>
+    <t>12/1</t>
+  </si>
+  <si>
+    <t>MP Interiores e Serv Ltda</t>
+  </si>
+  <si>
+    <t>R$  736,71</t>
+  </si>
+  <si>
+    <t>23/04/26</t>
+  </si>
+  <si>
+    <t>Digisac</t>
   </si>
   <si>
     <t>9/1</t>
@@ -1172,15 +1172,87 @@
     <t>4.02.02.01.01 Fretes sobre compra de mercadorias da marca - provisão</t>
   </si>
   <si>
+    <t>ENTREGADORA NOVO RUMO LTDA ME</t>
+  </si>
+  <si>
+    <t>R$  141,50</t>
+  </si>
+  <si>
+    <t>68501AMILTONF</t>
+  </si>
+  <si>
+    <t>63301n/0</t>
+  </si>
+  <si>
+    <t>R$  243,97</t>
+  </si>
+  <si>
+    <t>RODAG TRANSPORTES LTDA*</t>
+  </si>
+  <si>
+    <t>R$  11,98</t>
+  </si>
+  <si>
+    <t>R$  11,18</t>
+  </si>
+  <si>
+    <t>66301-/0</t>
+  </si>
+  <si>
+    <t>R$  101,41</t>
+  </si>
+  <si>
+    <t>67501-/0</t>
+  </si>
+  <si>
+    <t>R$  95,00</t>
+  </si>
+  <si>
+    <t>70601-/0</t>
+  </si>
+  <si>
+    <t>66301n/0</t>
+  </si>
+  <si>
+    <t>64801n/0</t>
+  </si>
+  <si>
+    <t>R$  190,00</t>
+  </si>
+  <si>
+    <t>R$  50,00</t>
+  </si>
+  <si>
+    <t>R$  98,75</t>
+  </si>
+  <si>
+    <t>64801R/0</t>
+  </si>
+  <si>
+    <t>R$  12,95</t>
+  </si>
+  <si>
+    <t>64801N/0</t>
+  </si>
+  <si>
+    <t>R$  12,09</t>
+  </si>
+  <si>
+    <t>63701/0</t>
+  </si>
+  <si>
+    <t>R$  14,09</t>
+  </si>
+  <si>
+    <t>R$  15,09</t>
+  </si>
+  <si>
     <t>67301/2</t>
   </si>
   <si>
     <t>PCP</t>
   </si>
   <si>
-    <t>ENTREGADORA NOVO RUMO LTDA ME</t>
-  </si>
-  <si>
     <t>R$  758,85</t>
   </si>
   <si>
@@ -1190,9 +1262,6 @@
     <t>67301/3</t>
   </si>
   <si>
-    <t>RODAG TRANSPORTES LTDA*</t>
-  </si>
-  <si>
     <t>R$  773,11</t>
   </si>
   <si>
@@ -1259,9 +1328,6 @@
     <t>R$  1.680,23</t>
   </si>
   <si>
-    <t>68501AMILTONF</t>
-  </si>
-  <si>
     <t>66301/2</t>
   </si>
   <si>
@@ -1358,9 +1424,6 @@
     <t>R$  264,04</t>
   </si>
   <si>
-    <t>67501-/0</t>
-  </si>
-  <si>
     <t>R$  136,00</t>
   </si>
   <si>
@@ -1373,9 +1436,6 @@
     <t>R$  33,33</t>
   </si>
   <si>
-    <t>R$  50,00</t>
-  </si>
-  <si>
     <t>R$  30,00</t>
   </si>
   <si>
@@ -1389,66 +1449,6 @@
   </si>
   <si>
     <t>R$  11,45</t>
-  </si>
-  <si>
-    <t>R$  141,50</t>
-  </si>
-  <si>
-    <t>63301n/0</t>
-  </si>
-  <si>
-    <t>R$  243,97</t>
-  </si>
-  <si>
-    <t>R$  11,98</t>
-  </si>
-  <si>
-    <t>R$  11,18</t>
-  </si>
-  <si>
-    <t>66301-/0</t>
-  </si>
-  <si>
-    <t>R$  101,41</t>
-  </si>
-  <si>
-    <t>R$  95,00</t>
-  </si>
-  <si>
-    <t>70601-/0</t>
-  </si>
-  <si>
-    <t>66301n/0</t>
-  </si>
-  <si>
-    <t>64801n/0</t>
-  </si>
-  <si>
-    <t>R$  190,00</t>
-  </si>
-  <si>
-    <t>R$  98,75</t>
-  </si>
-  <si>
-    <t>64801R/0</t>
-  </si>
-  <si>
-    <t>R$  12,95</t>
-  </si>
-  <si>
-    <t>64801N/0</t>
-  </si>
-  <si>
-    <t>R$  12,09</t>
-  </si>
-  <si>
-    <t>63701/0</t>
-  </si>
-  <si>
-    <t>R$  14,09</t>
-  </si>
-  <si>
-    <t>R$  15,09</t>
   </si>
   <si>
     <t>4.03 DESPESAS DE VENDAS</t>
@@ -2190,9 +2190,36 @@
     <t>R$ 9.161,99</t>
   </si>
   <si>
+    <t>WEBGIGA SOLUCOES DIGITAIS LTDA</t>
+  </si>
+  <si>
+    <t>R$  4.588,50</t>
+  </si>
+  <si>
+    <t>18/02/26</t>
+  </si>
+  <si>
+    <t>Webgiga 2026</t>
+  </si>
+  <si>
     <t>12/3</t>
   </si>
   <si>
+    <t>MARQUES MAIO MARKETING DIGITAL LTDA</t>
+  </si>
+  <si>
+    <t>R$  808,50</t>
+  </si>
+  <si>
+    <t>08/01/26</t>
+  </si>
+  <si>
+    <t>01/03/26</t>
+  </si>
+  <si>
+    <t>MHM - Honorários 2026</t>
+  </si>
+  <si>
     <t>Google</t>
   </si>
   <si>
@@ -2202,21 +2229,6 @@
     <t>Google 2026</t>
   </si>
   <si>
-    <t>MARQUES MAIO MARKETING DIGITAL LTDA</t>
-  </si>
-  <si>
-    <t>R$  808,50</t>
-  </si>
-  <si>
-    <t>08/01/26</t>
-  </si>
-  <si>
-    <t>01/03/26</t>
-  </si>
-  <si>
-    <t>MHM - Honorários 2026</t>
-  </si>
-  <si>
     <t>1/1</t>
   </si>
   <si>
@@ -2232,18 +2244,6 @@
     <t>Facebook 2026</t>
   </si>
   <si>
-    <t>WEBGIGA SOLUCOES DIGITAIS LTDA</t>
-  </si>
-  <si>
-    <t>R$  4.588,50</t>
-  </si>
-  <si>
-    <t>18/02/26</t>
-  </si>
-  <si>
-    <t>Webgiga 2026</t>
-  </si>
-  <si>
     <t>4.03.03.09.06 Marketing - outros gastos (CV)</t>
   </si>
   <si>
@@ -2643,6 +2643,18 @@
     <t>4.04.02.06.01 Material de escritório - uso e consumo</t>
   </si>
   <si>
+    <t>595/1</t>
+  </si>
+  <si>
+    <t>Oxxo</t>
+  </si>
+  <si>
+    <t>R$  110,94</t>
+  </si>
+  <si>
+    <t>Cafés loja</t>
+  </si>
+  <si>
     <t>593/1</t>
   </si>
   <si>
@@ -2659,18 +2671,6 @@
   </si>
   <si>
     <t>R$  19,98</t>
-  </si>
-  <si>
-    <t>595/1</t>
-  </si>
-  <si>
-    <t>Oxxo</t>
-  </si>
-  <si>
-    <t>R$  110,94</t>
-  </si>
-  <si>
-    <t>Cafés loja</t>
   </si>
   <si>
     <t>569/1</t>
@@ -2759,6 +2759,21 @@
     <t>4.04.02.08.03 Mensalidades e assinaturas - outros gastos</t>
   </si>
   <si>
+    <t>3/2</t>
+  </si>
+  <si>
+    <t>R$  1.248,76</t>
+  </si>
+  <si>
+    <t>Promob 2026/2</t>
+  </si>
+  <si>
+    <t>R$  599,00</t>
+  </si>
+  <si>
+    <t>Promob 2026</t>
+  </si>
+  <si>
     <t>592/1</t>
   </si>
   <si>
@@ -2777,21 +2792,6 @@
     <t>D4 sign 2026</t>
   </si>
   <si>
-    <t>R$  599,00</t>
-  </si>
-  <si>
-    <t>Promob 2026</t>
-  </si>
-  <si>
-    <t>3/2</t>
-  </si>
-  <si>
-    <t>R$  1.248,76</t>
-  </si>
-  <si>
-    <t>Promob 2026/2</t>
-  </si>
-  <si>
     <t>4.04.02.11 Manutenção de predio e equipamentos</t>
   </si>
   <si>
@@ -2858,6 +2858,15 @@
     <t>R$ 400,33</t>
   </si>
   <si>
+    <t>Jackson Fernando de Araujo</t>
+  </si>
+  <si>
+    <t>R$  150,00</t>
+  </si>
+  <si>
+    <t>Segurança 2026</t>
+  </si>
+  <si>
     <t>VERISURE</t>
   </si>
   <si>
@@ -2865,15 +2874,6 @@
   </si>
   <si>
     <t>Verisure - Alarme 2026</t>
-  </si>
-  <si>
-    <t>Jackson Fernando de Araujo</t>
-  </si>
-  <si>
-    <t>R$  150,00</t>
-  </si>
-  <si>
-    <t>Segurança 2026</t>
   </si>
   <si>
     <t>4.04.02.14.08 Site e newsletter da loja</t>
@@ -6040,13 +6040,13 @@
         <v>193</v>
       </c>
       <c r="J61" t="s">
+        <v>83</v>
+      </c>
+      <c r="K61" t="s">
+        <v>67</v>
+      </c>
+      <c r="L61" t="s">
         <v>194</v>
-      </c>
-      <c r="K61" t="s">
-        <v>133</v>
-      </c>
-      <c r="L61" t="s">
-        <v>195</v>
       </c>
       <c r="M61" t="s">
         <v>183</v>
@@ -6081,7 +6081,7 @@
         <v>34</v>
       </c>
       <c r="E62" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="F62" t="s">
         <v>64</v>
@@ -6090,16 +6090,16 @@
         <v>41</v>
       </c>
       <c r="H62" t="s">
+        <v>196</v>
+      </c>
+      <c r="I62" t="s">
         <v>197</v>
       </c>
-      <c r="I62" t="s">
+      <c r="J62" t="s">
         <v>198</v>
       </c>
-      <c r="J62" t="s">
-        <v>83</v>
-      </c>
       <c r="K62" t="s">
-        <v>67</v>
+        <v>133</v>
       </c>
       <c r="L62" t="s">
         <v>199</v>
@@ -6114,7 +6114,7 @@
         <v>48</v>
       </c>
       <c r="P62" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="Q62" t="s">
         <v>47</v>
@@ -6146,7 +6146,7 @@
         <v>41</v>
       </c>
       <c r="H63" t="s">
-        <v>197</v>
+        <v>192</v>
       </c>
       <c r="I63" t="s">
         <v>201</v>
@@ -6320,7 +6320,7 @@
         <v>210</v>
       </c>
       <c r="J66" t="s">
-        <v>194</v>
+        <v>198</v>
       </c>
       <c r="K66" t="s">
         <v>159</v>
@@ -9889,19 +9889,19 @@
         <v>33</v>
       </c>
       <c r="E130" t="s">
+        <v>87</v>
+      </c>
+      <c r="F130" t="s">
+        <v>208</v>
+      </c>
+      <c r="G130" t="s">
+        <v>41</v>
+      </c>
+      <c r="H130" t="s">
         <v>383</v>
       </c>
-      <c r="F130" t="s">
+      <c r="I130" t="s">
         <v>384</v>
-      </c>
-      <c r="G130" t="s">
-        <v>41</v>
-      </c>
-      <c r="H130" t="s">
-        <v>385</v>
-      </c>
-      <c r="I130" t="s">
-        <v>386</v>
       </c>
       <c r="J130" t="s">
         <v>73</v>
@@ -9910,7 +9910,7 @@
         <v>73</v>
       </c>
       <c r="L130" t="s">
-        <v>387</v>
+        <v>34</v>
       </c>
       <c r="M130" t="s">
         <v>382</v>
@@ -9919,13 +9919,13 @@
         <v>47</v>
       </c>
       <c r="O130" t="s">
-        <v>34</v>
+        <v>385</v>
       </c>
       <c r="P130" t="s">
-        <v>34</v>
+        <v>384</v>
       </c>
       <c r="Q130" t="s">
-        <v>34</v>
+        <v>47</v>
       </c>
       <c r="R130" t="s">
         <v>34</v>
@@ -9945,28 +9945,28 @@
         <v>34</v>
       </c>
       <c r="E131" t="s">
-        <v>388</v>
+        <v>386</v>
       </c>
       <c r="F131" t="s">
-        <v>384</v>
+        <v>208</v>
       </c>
       <c r="G131" t="s">
         <v>41</v>
       </c>
       <c r="H131" t="s">
-        <v>389</v>
+        <v>383</v>
       </c>
       <c r="I131" t="s">
-        <v>390</v>
+        <v>387</v>
       </c>
       <c r="J131" t="s">
-        <v>73</v>
+        <v>97</v>
       </c>
       <c r="K131" t="s">
-        <v>73</v>
+        <v>97</v>
       </c>
       <c r="L131" t="s">
-        <v>387</v>
+        <v>34</v>
       </c>
       <c r="M131" t="s">
         <v>382</v>
@@ -9975,13 +9975,13 @@
         <v>47</v>
       </c>
       <c r="O131" t="s">
-        <v>34</v>
+        <v>98</v>
       </c>
       <c r="P131" t="s">
-        <v>34</v>
+        <v>387</v>
       </c>
       <c r="Q131" t="s">
-        <v>34</v>
+        <v>47</v>
       </c>
       <c r="R131" t="s">
         <v>34</v>
@@ -10001,28 +10001,28 @@
         <v>34</v>
       </c>
       <c r="E132" t="s">
-        <v>391</v>
+        <v>113</v>
       </c>
       <c r="F132" t="s">
-        <v>384</v>
+        <v>208</v>
       </c>
       <c r="G132" t="s">
         <v>41</v>
       </c>
       <c r="H132" t="s">
-        <v>385</v>
+        <v>388</v>
       </c>
       <c r="I132" t="s">
-        <v>392</v>
+        <v>389</v>
       </c>
       <c r="J132" t="s">
-        <v>165</v>
+        <v>73</v>
       </c>
       <c r="K132" t="s">
-        <v>165</v>
+        <v>73</v>
       </c>
       <c r="L132" t="s">
-        <v>387</v>
+        <v>34</v>
       </c>
       <c r="M132" t="s">
         <v>382</v>
@@ -10031,13 +10031,13 @@
         <v>47</v>
       </c>
       <c r="O132" t="s">
-        <v>34</v>
+        <v>115</v>
       </c>
       <c r="P132" t="s">
-        <v>34</v>
+        <v>389</v>
       </c>
       <c r="Q132" t="s">
-        <v>34</v>
+        <v>47</v>
       </c>
       <c r="R132" t="s">
         <v>34</v>
@@ -10057,28 +10057,28 @@
         <v>34</v>
       </c>
       <c r="E133" t="s">
-        <v>393</v>
+        <v>113</v>
       </c>
       <c r="F133" t="s">
-        <v>384</v>
+        <v>208</v>
       </c>
       <c r="G133" t="s">
         <v>41</v>
       </c>
       <c r="H133" t="s">
-        <v>389</v>
+        <v>383</v>
       </c>
       <c r="I133" t="s">
-        <v>394</v>
+        <v>390</v>
       </c>
       <c r="J133" t="s">
-        <v>165</v>
+        <v>73</v>
       </c>
       <c r="K133" t="s">
-        <v>165</v>
+        <v>73</v>
       </c>
       <c r="L133" t="s">
-        <v>387</v>
+        <v>34</v>
       </c>
       <c r="M133" t="s">
         <v>382</v>
@@ -10087,13 +10087,13 @@
         <v>47</v>
       </c>
       <c r="O133" t="s">
-        <v>34</v>
+        <v>115</v>
       </c>
       <c r="P133" t="s">
-        <v>34</v>
+        <v>390</v>
       </c>
       <c r="Q133" t="s">
-        <v>34</v>
+        <v>47</v>
       </c>
       <c r="R133" t="s">
         <v>34</v>
@@ -10113,28 +10113,28 @@
         <v>34</v>
       </c>
       <c r="E134" t="s">
-        <v>395</v>
+        <v>391</v>
       </c>
       <c r="F134" t="s">
-        <v>247</v>
+        <v>208</v>
       </c>
       <c r="G134" t="s">
         <v>41</v>
       </c>
       <c r="H134" t="s">
-        <v>389</v>
+        <v>383</v>
       </c>
       <c r="I134" t="s">
-        <v>396</v>
+        <v>392</v>
       </c>
       <c r="J134" t="s">
-        <v>73</v>
+        <v>68</v>
       </c>
       <c r="K134" t="s">
-        <v>73</v>
+        <v>68</v>
       </c>
       <c r="L134" t="s">
-        <v>387</v>
+        <v>34</v>
       </c>
       <c r="M134" t="s">
         <v>382</v>
@@ -10143,10 +10143,10 @@
         <v>47</v>
       </c>
       <c r="O134" t="s">
-        <v>115</v>
+        <v>262</v>
       </c>
       <c r="P134" t="s">
-        <v>396</v>
+        <v>392</v>
       </c>
       <c r="Q134" t="s">
         <v>47</v>
@@ -10169,28 +10169,28 @@
         <v>34</v>
       </c>
       <c r="E135" t="s">
-        <v>397</v>
+        <v>393</v>
       </c>
       <c r="F135" t="s">
-        <v>247</v>
+        <v>208</v>
       </c>
       <c r="G135" t="s">
         <v>41</v>
       </c>
       <c r="H135" t="s">
-        <v>385</v>
+        <v>383</v>
       </c>
       <c r="I135" t="s">
-        <v>398</v>
+        <v>394</v>
       </c>
       <c r="J135" t="s">
-        <v>105</v>
+        <v>119</v>
       </c>
       <c r="K135" t="s">
-        <v>105</v>
+        <v>119</v>
       </c>
       <c r="L135" t="s">
-        <v>387</v>
+        <v>34</v>
       </c>
       <c r="M135" t="s">
         <v>382</v>
@@ -10199,10 +10199,10 @@
         <v>47</v>
       </c>
       <c r="O135" t="s">
-        <v>112</v>
+        <v>269</v>
       </c>
       <c r="P135" t="s">
-        <v>398</v>
+        <v>394</v>
       </c>
       <c r="Q135" t="s">
         <v>47</v>
@@ -10225,28 +10225,28 @@
         <v>34</v>
       </c>
       <c r="E136" t="s">
-        <v>300</v>
+        <v>395</v>
       </c>
       <c r="F136" t="s">
-        <v>247</v>
+        <v>208</v>
       </c>
       <c r="G136" t="s">
         <v>41</v>
       </c>
       <c r="H136" t="s">
-        <v>385</v>
+        <v>383</v>
       </c>
       <c r="I136" t="s">
-        <v>399</v>
+        <v>394</v>
       </c>
       <c r="J136" t="s">
-        <v>97</v>
+        <v>78</v>
       </c>
       <c r="K136" t="s">
-        <v>97</v>
+        <v>78</v>
       </c>
       <c r="L136" t="s">
-        <v>387</v>
+        <v>34</v>
       </c>
       <c r="M136" t="s">
         <v>382</v>
@@ -10255,10 +10255,10 @@
         <v>47</v>
       </c>
       <c r="O136" t="s">
-        <v>98</v>
+        <v>169</v>
       </c>
       <c r="P136" t="s">
-        <v>399</v>
+        <v>394</v>
       </c>
       <c r="Q136" t="s">
         <v>47</v>
@@ -10281,28 +10281,28 @@
         <v>34</v>
       </c>
       <c r="E137" t="s">
-        <v>333</v>
+        <v>396</v>
       </c>
       <c r="F137" t="s">
-        <v>247</v>
+        <v>208</v>
       </c>
       <c r="G137" t="s">
         <v>41</v>
       </c>
       <c r="H137" t="s">
-        <v>385</v>
+        <v>383</v>
       </c>
       <c r="I137" t="s">
-        <v>400</v>
+        <v>394</v>
       </c>
       <c r="J137" t="s">
-        <v>73</v>
+        <v>68</v>
       </c>
       <c r="K137" t="s">
-        <v>73</v>
+        <v>68</v>
       </c>
       <c r="L137" t="s">
-        <v>387</v>
+        <v>34</v>
       </c>
       <c r="M137" t="s">
         <v>382</v>
@@ -10311,10 +10311,10 @@
         <v>47</v>
       </c>
       <c r="O137" t="s">
-        <v>330</v>
+        <v>262</v>
       </c>
       <c r="P137" t="s">
-        <v>400</v>
+        <v>394</v>
       </c>
       <c r="Q137" t="s">
         <v>47</v>
@@ -10337,28 +10337,28 @@
         <v>34</v>
       </c>
       <c r="E138" t="s">
-        <v>285</v>
+        <v>397</v>
       </c>
       <c r="F138" t="s">
-        <v>247</v>
+        <v>208</v>
       </c>
       <c r="G138" t="s">
         <v>41</v>
       </c>
       <c r="H138" t="s">
-        <v>389</v>
+        <v>383</v>
       </c>
       <c r="I138" t="s">
-        <v>401</v>
+        <v>398</v>
       </c>
       <c r="J138" t="s">
-        <v>68</v>
+        <v>73</v>
       </c>
       <c r="K138" t="s">
-        <v>68</v>
+        <v>73</v>
       </c>
       <c r="L138" t="s">
-        <v>387</v>
+        <v>34</v>
       </c>
       <c r="M138" t="s">
         <v>382</v>
@@ -10367,10 +10367,10 @@
         <v>47</v>
       </c>
       <c r="O138" t="s">
-        <v>262</v>
+        <v>115</v>
       </c>
       <c r="P138" t="s">
-        <v>401</v>
+        <v>398</v>
       </c>
       <c r="Q138" t="s">
         <v>47</v>
@@ -10393,28 +10393,28 @@
         <v>34</v>
       </c>
       <c r="E139" t="s">
-        <v>331</v>
+        <v>150</v>
       </c>
       <c r="F139" t="s">
-        <v>247</v>
+        <v>208</v>
       </c>
       <c r="G139" t="s">
         <v>41</v>
       </c>
       <c r="H139" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
       <c r="I139" t="s">
-        <v>402</v>
+        <v>399</v>
       </c>
       <c r="J139" t="s">
-        <v>73</v>
+        <v>120</v>
       </c>
       <c r="K139" t="s">
-        <v>73</v>
+        <v>120</v>
       </c>
       <c r="L139" t="s">
-        <v>387</v>
+        <v>34</v>
       </c>
       <c r="M139" t="s">
         <v>382</v>
@@ -10423,10 +10423,10 @@
         <v>47</v>
       </c>
       <c r="O139" t="s">
-        <v>330</v>
+        <v>152</v>
       </c>
       <c r="P139" t="s">
-        <v>402</v>
+        <v>399</v>
       </c>
       <c r="Q139" t="s">
         <v>47</v>
@@ -10449,28 +10449,28 @@
         <v>34</v>
       </c>
       <c r="E140" t="s">
-        <v>308</v>
+        <v>110</v>
       </c>
       <c r="F140" t="s">
-        <v>247</v>
+        <v>208</v>
       </c>
       <c r="G140" t="s">
         <v>41</v>
       </c>
       <c r="H140" t="s">
-        <v>389</v>
+        <v>383</v>
       </c>
       <c r="I140" t="s">
-        <v>403</v>
+        <v>400</v>
       </c>
       <c r="J140" t="s">
-        <v>119</v>
+        <v>105</v>
       </c>
       <c r="K140" t="s">
-        <v>119</v>
+        <v>105</v>
       </c>
       <c r="L140" t="s">
-        <v>387</v>
+        <v>34</v>
       </c>
       <c r="M140" t="s">
         <v>382</v>
@@ -10479,10 +10479,10 @@
         <v>47</v>
       </c>
       <c r="O140" t="s">
-        <v>269</v>
+        <v>112</v>
       </c>
       <c r="P140" t="s">
-        <v>403</v>
+        <v>400</v>
       </c>
       <c r="Q140" t="s">
         <v>47</v>
@@ -10505,28 +10505,28 @@
         <v>34</v>
       </c>
       <c r="E141" t="s">
-        <v>306</v>
+        <v>401</v>
       </c>
       <c r="F141" t="s">
-        <v>247</v>
+        <v>208</v>
       </c>
       <c r="G141" t="s">
         <v>41</v>
       </c>
       <c r="H141" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
       <c r="I141" t="s">
-        <v>404</v>
+        <v>402</v>
       </c>
       <c r="J141" t="s">
-        <v>97</v>
+        <v>73</v>
       </c>
       <c r="K141" t="s">
-        <v>97</v>
+        <v>73</v>
       </c>
       <c r="L141" t="s">
-        <v>387</v>
+        <v>34</v>
       </c>
       <c r="M141" t="s">
         <v>382</v>
@@ -10535,10 +10535,10 @@
         <v>47</v>
       </c>
       <c r="O141" t="s">
-        <v>98</v>
+        <v>115</v>
       </c>
       <c r="P141" t="s">
-        <v>404</v>
+        <v>402</v>
       </c>
       <c r="Q141" t="s">
         <v>47</v>
@@ -10561,28 +10561,28 @@
         <v>34</v>
       </c>
       <c r="E142" t="s">
-        <v>405</v>
+        <v>150</v>
       </c>
       <c r="F142" t="s">
-        <v>247</v>
+        <v>208</v>
       </c>
       <c r="G142" t="s">
         <v>41</v>
       </c>
       <c r="H142" t="s">
-        <v>385</v>
+        <v>383</v>
       </c>
       <c r="I142" t="s">
-        <v>406</v>
+        <v>394</v>
       </c>
       <c r="J142" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="K142" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="L142" t="s">
-        <v>387</v>
+        <v>34</v>
       </c>
       <c r="M142" t="s">
         <v>382</v>
@@ -10591,10 +10591,10 @@
         <v>47</v>
       </c>
       <c r="O142" t="s">
-        <v>269</v>
+        <v>152</v>
       </c>
       <c r="P142" t="s">
-        <v>406</v>
+        <v>394</v>
       </c>
       <c r="Q142" t="s">
         <v>47</v>
@@ -10617,28 +10617,28 @@
         <v>34</v>
       </c>
       <c r="E143" t="s">
-        <v>407</v>
+        <v>403</v>
       </c>
       <c r="F143" t="s">
-        <v>247</v>
+        <v>208</v>
       </c>
       <c r="G143" t="s">
         <v>41</v>
       </c>
       <c r="H143" t="s">
-        <v>389</v>
+        <v>383</v>
       </c>
       <c r="I143" t="s">
-        <v>408</v>
+        <v>404</v>
       </c>
       <c r="J143" t="s">
-        <v>78</v>
+        <v>73</v>
       </c>
       <c r="K143" t="s">
-        <v>78</v>
+        <v>73</v>
       </c>
       <c r="L143" t="s">
-        <v>387</v>
+        <v>34</v>
       </c>
       <c r="M143" t="s">
         <v>382</v>
@@ -10647,10 +10647,10 @@
         <v>47</v>
       </c>
       <c r="O143" t="s">
-        <v>169</v>
+        <v>115</v>
       </c>
       <c r="P143" t="s">
-        <v>408</v>
+        <v>404</v>
       </c>
       <c r="Q143" t="s">
         <v>47</v>
@@ -10673,28 +10673,28 @@
         <v>34</v>
       </c>
       <c r="E144" t="s">
-        <v>409</v>
+        <v>405</v>
       </c>
       <c r="F144" t="s">
-        <v>247</v>
+        <v>208</v>
       </c>
       <c r="G144" t="s">
         <v>41</v>
       </c>
       <c r="H144" t="s">
-        <v>389</v>
+        <v>383</v>
       </c>
       <c r="I144" t="s">
-        <v>410</v>
+        <v>406</v>
       </c>
       <c r="J144" t="s">
-        <v>119</v>
+        <v>73</v>
       </c>
       <c r="K144" t="s">
-        <v>119</v>
+        <v>73</v>
       </c>
       <c r="L144" t="s">
-        <v>387</v>
+        <v>34</v>
       </c>
       <c r="M144" t="s">
         <v>382</v>
@@ -10703,10 +10703,10 @@
         <v>47</v>
       </c>
       <c r="O144" t="s">
-        <v>149</v>
+        <v>294</v>
       </c>
       <c r="P144" t="s">
-        <v>410</v>
+        <v>406</v>
       </c>
       <c r="Q144" t="s">
         <v>47</v>
@@ -10729,19 +10729,19 @@
         <v>34</v>
       </c>
       <c r="E145" t="s">
-        <v>312</v>
+        <v>405</v>
       </c>
       <c r="F145" t="s">
-        <v>247</v>
+        <v>208</v>
       </c>
       <c r="G145" t="s">
         <v>41</v>
       </c>
       <c r="H145" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
       <c r="I145" t="s">
-        <v>411</v>
+        <v>407</v>
       </c>
       <c r="J145" t="s">
         <v>73</v>
@@ -10750,7 +10750,7 @@
         <v>73</v>
       </c>
       <c r="L145" t="s">
-        <v>387</v>
+        <v>34</v>
       </c>
       <c r="M145" t="s">
         <v>382</v>
@@ -10759,10 +10759,10 @@
         <v>47</v>
       </c>
       <c r="O145" t="s">
-        <v>412</v>
+        <v>294</v>
       </c>
       <c r="P145" t="s">
-        <v>411</v>
+        <v>407</v>
       </c>
       <c r="Q145" t="s">
         <v>47</v>
@@ -10785,28 +10785,28 @@
         <v>34</v>
       </c>
       <c r="E146" t="s">
-        <v>413</v>
+        <v>408</v>
       </c>
       <c r="F146" t="s">
-        <v>247</v>
+        <v>409</v>
       </c>
       <c r="G146" t="s">
         <v>41</v>
       </c>
       <c r="H146" t="s">
-        <v>385</v>
+        <v>383</v>
       </c>
       <c r="I146" t="s">
-        <v>414</v>
+        <v>410</v>
       </c>
       <c r="J146" t="s">
-        <v>68</v>
+        <v>73</v>
       </c>
       <c r="K146" t="s">
-        <v>68</v>
+        <v>73</v>
       </c>
       <c r="L146" t="s">
-        <v>387</v>
+        <v>411</v>
       </c>
       <c r="M146" t="s">
         <v>382</v>
@@ -10815,13 +10815,13 @@
         <v>47</v>
       </c>
       <c r="O146" t="s">
-        <v>262</v>
+        <v>34</v>
       </c>
       <c r="P146" t="s">
-        <v>414</v>
+        <v>34</v>
       </c>
       <c r="Q146" t="s">
-        <v>47</v>
+        <v>34</v>
       </c>
       <c r="R146" t="s">
         <v>34</v>
@@ -10841,28 +10841,28 @@
         <v>34</v>
       </c>
       <c r="E147" t="s">
-        <v>276</v>
+        <v>412</v>
       </c>
       <c r="F147" t="s">
-        <v>247</v>
+        <v>409</v>
       </c>
       <c r="G147" t="s">
         <v>41</v>
       </c>
       <c r="H147" t="s">
-        <v>385</v>
+        <v>388</v>
       </c>
       <c r="I147" t="s">
-        <v>415</v>
+        <v>413</v>
       </c>
       <c r="J147" t="s">
-        <v>78</v>
+        <v>73</v>
       </c>
       <c r="K147" t="s">
-        <v>78</v>
+        <v>73</v>
       </c>
       <c r="L147" t="s">
-        <v>387</v>
+        <v>411</v>
       </c>
       <c r="M147" t="s">
         <v>382</v>
@@ -10871,13 +10871,13 @@
         <v>47</v>
       </c>
       <c r="O147" t="s">
-        <v>169</v>
+        <v>34</v>
       </c>
       <c r="P147" t="s">
-        <v>415</v>
+        <v>34</v>
       </c>
       <c r="Q147" t="s">
-        <v>47</v>
+        <v>34</v>
       </c>
       <c r="R147" t="s">
         <v>34</v>
@@ -10897,28 +10897,28 @@
         <v>34</v>
       </c>
       <c r="E148" t="s">
-        <v>416</v>
+        <v>414</v>
       </c>
       <c r="F148" t="s">
-        <v>247</v>
+        <v>409</v>
       </c>
       <c r="G148" t="s">
         <v>41</v>
       </c>
       <c r="H148" t="s">
-        <v>385</v>
+        <v>383</v>
       </c>
       <c r="I148" t="s">
-        <v>417</v>
+        <v>415</v>
       </c>
       <c r="J148" t="s">
-        <v>73</v>
+        <v>165</v>
       </c>
       <c r="K148" t="s">
-        <v>73</v>
+        <v>165</v>
       </c>
       <c r="L148" t="s">
-        <v>387</v>
+        <v>411</v>
       </c>
       <c r="M148" t="s">
         <v>382</v>
@@ -10927,13 +10927,13 @@
         <v>47</v>
       </c>
       <c r="O148" t="s">
-        <v>412</v>
+        <v>34</v>
       </c>
       <c r="P148" t="s">
-        <v>417</v>
+        <v>34</v>
       </c>
       <c r="Q148" t="s">
-        <v>47</v>
+        <v>34</v>
       </c>
       <c r="R148" t="s">
         <v>34</v>
@@ -10953,28 +10953,28 @@
         <v>34</v>
       </c>
       <c r="E149" t="s">
-        <v>303</v>
+        <v>416</v>
       </c>
       <c r="F149" t="s">
-        <v>247</v>
+        <v>409</v>
       </c>
       <c r="G149" t="s">
         <v>41</v>
       </c>
       <c r="H149" t="s">
-        <v>385</v>
+        <v>388</v>
       </c>
       <c r="I149" t="s">
-        <v>418</v>
+        <v>417</v>
       </c>
       <c r="J149" t="s">
-        <v>119</v>
+        <v>165</v>
       </c>
       <c r="K149" t="s">
-        <v>119</v>
+        <v>165</v>
       </c>
       <c r="L149" t="s">
-        <v>387</v>
+        <v>411</v>
       </c>
       <c r="M149" t="s">
         <v>382</v>
@@ -10983,13 +10983,13 @@
         <v>47</v>
       </c>
       <c r="O149" t="s">
-        <v>149</v>
+        <v>34</v>
       </c>
       <c r="P149" t="s">
-        <v>418</v>
+        <v>34</v>
       </c>
       <c r="Q149" t="s">
-        <v>47</v>
+        <v>34</v>
       </c>
       <c r="R149" t="s">
         <v>34</v>
@@ -11009,7 +11009,7 @@
         <v>34</v>
       </c>
       <c r="E150" t="s">
-        <v>298</v>
+        <v>418</v>
       </c>
       <c r="F150" t="s">
         <v>247</v>
@@ -11018,7 +11018,7 @@
         <v>41</v>
       </c>
       <c r="H150" t="s">
-        <v>385</v>
+        <v>388</v>
       </c>
       <c r="I150" t="s">
         <v>419</v>
@@ -11030,7 +11030,7 @@
         <v>73</v>
       </c>
       <c r="L150" t="s">
-        <v>387</v>
+        <v>411</v>
       </c>
       <c r="M150" t="s">
         <v>382</v>
@@ -11074,19 +11074,19 @@
         <v>41</v>
       </c>
       <c r="H151" t="s">
-        <v>389</v>
+        <v>383</v>
       </c>
       <c r="I151" t="s">
         <v>421</v>
       </c>
       <c r="J151" t="s">
-        <v>133</v>
+        <v>105</v>
       </c>
       <c r="K151" t="s">
-        <v>133</v>
+        <v>105</v>
       </c>
       <c r="L151" t="s">
-        <v>387</v>
+        <v>411</v>
       </c>
       <c r="M151" t="s">
         <v>382</v>
@@ -11095,7 +11095,7 @@
         <v>47</v>
       </c>
       <c r="O151" t="s">
-        <v>145</v>
+        <v>112</v>
       </c>
       <c r="P151" t="s">
         <v>421</v>
@@ -11121,7 +11121,7 @@
         <v>34</v>
       </c>
       <c r="E152" t="s">
-        <v>422</v>
+        <v>300</v>
       </c>
       <c r="F152" t="s">
         <v>247</v>
@@ -11130,19 +11130,19 @@
         <v>41</v>
       </c>
       <c r="H152" t="s">
-        <v>389</v>
+        <v>383</v>
       </c>
       <c r="I152" t="s">
-        <v>423</v>
+        <v>422</v>
       </c>
       <c r="J152" t="s">
-        <v>105</v>
+        <v>97</v>
       </c>
       <c r="K152" t="s">
-        <v>105</v>
+        <v>97</v>
       </c>
       <c r="L152" t="s">
-        <v>387</v>
+        <v>411</v>
       </c>
       <c r="M152" t="s">
         <v>382</v>
@@ -11151,10 +11151,10 @@
         <v>47</v>
       </c>
       <c r="O152" t="s">
-        <v>112</v>
+        <v>98</v>
       </c>
       <c r="P152" t="s">
-        <v>423</v>
+        <v>422</v>
       </c>
       <c r="Q152" t="s">
         <v>47</v>
@@ -11177,7 +11177,7 @@
         <v>34</v>
       </c>
       <c r="E153" t="s">
-        <v>424</v>
+        <v>333</v>
       </c>
       <c r="F153" t="s">
         <v>247</v>
@@ -11186,19 +11186,19 @@
         <v>41</v>
       </c>
       <c r="H153" t="s">
-        <v>385</v>
+        <v>383</v>
       </c>
       <c r="I153" t="s">
-        <v>425</v>
+        <v>423</v>
       </c>
       <c r="J153" t="s">
-        <v>120</v>
+        <v>73</v>
       </c>
       <c r="K153" t="s">
-        <v>120</v>
+        <v>73</v>
       </c>
       <c r="L153" t="s">
-        <v>387</v>
+        <v>411</v>
       </c>
       <c r="M153" t="s">
         <v>382</v>
@@ -11207,10 +11207,10 @@
         <v>47</v>
       </c>
       <c r="O153" t="s">
-        <v>152</v>
+        <v>330</v>
       </c>
       <c r="P153" t="s">
-        <v>425</v>
+        <v>423</v>
       </c>
       <c r="Q153" t="s">
         <v>47</v>
@@ -11233,7 +11233,7 @@
         <v>34</v>
       </c>
       <c r="E154" t="s">
-        <v>426</v>
+        <v>285</v>
       </c>
       <c r="F154" t="s">
         <v>247</v>
@@ -11242,19 +11242,19 @@
         <v>41</v>
       </c>
       <c r="H154" t="s">
-        <v>385</v>
+        <v>388</v>
       </c>
       <c r="I154" t="s">
-        <v>427</v>
+        <v>424</v>
       </c>
       <c r="J154" t="s">
-        <v>73</v>
+        <v>68</v>
       </c>
       <c r="K154" t="s">
-        <v>73</v>
+        <v>68</v>
       </c>
       <c r="L154" t="s">
-        <v>387</v>
+        <v>411</v>
       </c>
       <c r="M154" t="s">
         <v>382</v>
@@ -11263,10 +11263,10 @@
         <v>47</v>
       </c>
       <c r="O154" t="s">
-        <v>294</v>
+        <v>262</v>
       </c>
       <c r="P154" t="s">
-        <v>427</v>
+        <v>424</v>
       </c>
       <c r="Q154" t="s">
         <v>47</v>
@@ -11289,7 +11289,7 @@
         <v>34</v>
       </c>
       <c r="E155" t="s">
-        <v>280</v>
+        <v>331</v>
       </c>
       <c r="F155" t="s">
         <v>247</v>
@@ -11298,19 +11298,19 @@
         <v>41</v>
       </c>
       <c r="H155" t="s">
-        <v>385</v>
+        <v>388</v>
       </c>
       <c r="I155" t="s">
-        <v>428</v>
+        <v>425</v>
       </c>
       <c r="J155" t="s">
-        <v>133</v>
+        <v>73</v>
       </c>
       <c r="K155" t="s">
-        <v>133</v>
+        <v>73</v>
       </c>
       <c r="L155" t="s">
-        <v>387</v>
+        <v>411</v>
       </c>
       <c r="M155" t="s">
         <v>382</v>
@@ -11319,10 +11319,10 @@
         <v>47</v>
       </c>
       <c r="O155" t="s">
-        <v>145</v>
+        <v>330</v>
       </c>
       <c r="P155" t="s">
-        <v>428</v>
+        <v>425</v>
       </c>
       <c r="Q155" t="s">
         <v>47</v>
@@ -11345,7 +11345,7 @@
         <v>34</v>
       </c>
       <c r="E156" t="s">
-        <v>429</v>
+        <v>308</v>
       </c>
       <c r="F156" t="s">
         <v>247</v>
@@ -11354,19 +11354,19 @@
         <v>41</v>
       </c>
       <c r="H156" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
       <c r="I156" t="s">
-        <v>430</v>
+        <v>426</v>
       </c>
       <c r="J156" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="K156" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="L156" t="s">
-        <v>387</v>
+        <v>411</v>
       </c>
       <c r="M156" t="s">
         <v>382</v>
@@ -11375,10 +11375,10 @@
         <v>47</v>
       </c>
       <c r="O156" t="s">
-        <v>152</v>
+        <v>269</v>
       </c>
       <c r="P156" t="s">
-        <v>430</v>
+        <v>426</v>
       </c>
       <c r="Q156" t="s">
         <v>47</v>
@@ -11401,7 +11401,7 @@
         <v>34</v>
       </c>
       <c r="E157" t="s">
-        <v>431</v>
+        <v>306</v>
       </c>
       <c r="F157" t="s">
         <v>247</v>
@@ -11410,19 +11410,19 @@
         <v>41</v>
       </c>
       <c r="H157" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
       <c r="I157" t="s">
-        <v>432</v>
+        <v>427</v>
       </c>
       <c r="J157" t="s">
-        <v>73</v>
+        <v>97</v>
       </c>
       <c r="K157" t="s">
-        <v>73</v>
+        <v>97</v>
       </c>
       <c r="L157" t="s">
-        <v>387</v>
+        <v>411</v>
       </c>
       <c r="M157" t="s">
         <v>382</v>
@@ -11431,10 +11431,10 @@
         <v>47</v>
       </c>
       <c r="O157" t="s">
-        <v>294</v>
+        <v>98</v>
       </c>
       <c r="P157" t="s">
-        <v>432</v>
+        <v>427</v>
       </c>
       <c r="Q157" t="s">
         <v>47</v>
@@ -11457,28 +11457,28 @@
         <v>34</v>
       </c>
       <c r="E158" t="s">
-        <v>433</v>
+        <v>428</v>
       </c>
       <c r="F158" t="s">
-        <v>208</v>
+        <v>247</v>
       </c>
       <c r="G158" t="s">
         <v>41</v>
       </c>
       <c r="H158" t="s">
-        <v>389</v>
+        <v>383</v>
       </c>
       <c r="I158" t="s">
-        <v>434</v>
+        <v>429</v>
       </c>
       <c r="J158" t="s">
-        <v>45</v>
+        <v>119</v>
       </c>
       <c r="K158" t="s">
-        <v>45</v>
+        <v>119</v>
       </c>
       <c r="L158" t="s">
-        <v>34</v>
+        <v>411</v>
       </c>
       <c r="M158" t="s">
         <v>382</v>
@@ -11487,10 +11487,10 @@
         <v>47</v>
       </c>
       <c r="O158" t="s">
-        <v>48</v>
+        <v>269</v>
       </c>
       <c r="P158" t="s">
-        <v>434</v>
+        <v>429</v>
       </c>
       <c r="Q158" t="s">
         <v>47</v>
@@ -11513,28 +11513,28 @@
         <v>34</v>
       </c>
       <c r="E159" t="s">
-        <v>435</v>
+        <v>430</v>
       </c>
       <c r="F159" t="s">
-        <v>208</v>
+        <v>247</v>
       </c>
       <c r="G159" t="s">
         <v>41</v>
       </c>
       <c r="H159" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
       <c r="I159" t="s">
-        <v>436</v>
+        <v>431</v>
       </c>
       <c r="J159" t="s">
-        <v>45</v>
+        <v>78</v>
       </c>
       <c r="K159" t="s">
-        <v>45</v>
+        <v>78</v>
       </c>
       <c r="L159" t="s">
-        <v>34</v>
+        <v>411</v>
       </c>
       <c r="M159" t="s">
         <v>382</v>
@@ -11543,10 +11543,10 @@
         <v>47</v>
       </c>
       <c r="O159" t="s">
-        <v>437</v>
+        <v>169</v>
       </c>
       <c r="P159" t="s">
-        <v>436</v>
+        <v>431</v>
       </c>
       <c r="Q159" t="s">
         <v>47</v>
@@ -11569,28 +11569,28 @@
         <v>34</v>
       </c>
       <c r="E160" t="s">
-        <v>94</v>
+        <v>432</v>
       </c>
       <c r="F160" t="s">
-        <v>208</v>
+        <v>247</v>
       </c>
       <c r="G160" t="s">
         <v>41</v>
       </c>
       <c r="H160" t="s">
-        <v>385</v>
+        <v>388</v>
       </c>
       <c r="I160" t="s">
-        <v>438</v>
+        <v>433</v>
       </c>
       <c r="J160" t="s">
-        <v>439</v>
+        <v>119</v>
       </c>
       <c r="K160" t="s">
-        <v>97</v>
+        <v>119</v>
       </c>
       <c r="L160" t="s">
-        <v>34</v>
+        <v>411</v>
       </c>
       <c r="M160" t="s">
         <v>382</v>
@@ -11599,10 +11599,10 @@
         <v>47</v>
       </c>
       <c r="O160" t="s">
-        <v>98</v>
+        <v>149</v>
       </c>
       <c r="P160" t="s">
-        <v>438</v>
+        <v>433</v>
       </c>
       <c r="Q160" t="s">
         <v>47</v>
@@ -11625,28 +11625,28 @@
         <v>34</v>
       </c>
       <c r="E161" t="s">
-        <v>440</v>
+        <v>312</v>
       </c>
       <c r="F161" t="s">
-        <v>208</v>
+        <v>247</v>
       </c>
       <c r="G161" t="s">
         <v>41</v>
       </c>
       <c r="H161" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
       <c r="I161" t="s">
-        <v>441</v>
+        <v>434</v>
       </c>
       <c r="J161" t="s">
-        <v>442</v>
+        <v>73</v>
       </c>
       <c r="K161" t="s">
-        <v>119</v>
+        <v>73</v>
       </c>
       <c r="L161" t="s">
-        <v>34</v>
+        <v>411</v>
       </c>
       <c r="M161" t="s">
         <v>382</v>
@@ -11655,10 +11655,10 @@
         <v>47</v>
       </c>
       <c r="O161" t="s">
-        <v>269</v>
+        <v>385</v>
       </c>
       <c r="P161" t="s">
-        <v>441</v>
+        <v>434</v>
       </c>
       <c r="Q161" t="s">
         <v>47</v>
@@ -11681,28 +11681,28 @@
         <v>34</v>
       </c>
       <c r="E162" t="s">
-        <v>94</v>
+        <v>435</v>
       </c>
       <c r="F162" t="s">
-        <v>208</v>
+        <v>247</v>
       </c>
       <c r="G162" t="s">
         <v>41</v>
       </c>
       <c r="H162" t="s">
-        <v>389</v>
+        <v>383</v>
       </c>
       <c r="I162" t="s">
-        <v>443</v>
+        <v>436</v>
       </c>
       <c r="J162" t="s">
-        <v>97</v>
+        <v>68</v>
       </c>
       <c r="K162" t="s">
-        <v>97</v>
+        <v>68</v>
       </c>
       <c r="L162" t="s">
-        <v>34</v>
+        <v>411</v>
       </c>
       <c r="M162" t="s">
         <v>382</v>
@@ -11711,10 +11711,10 @@
         <v>47</v>
       </c>
       <c r="O162" t="s">
-        <v>98</v>
+        <v>262</v>
       </c>
       <c r="P162" t="s">
-        <v>443</v>
+        <v>436</v>
       </c>
       <c r="Q162" t="s">
         <v>47</v>
@@ -11737,28 +11737,28 @@
         <v>34</v>
       </c>
       <c r="E163" t="s">
-        <v>440</v>
+        <v>276</v>
       </c>
       <c r="F163" t="s">
-        <v>208</v>
+        <v>247</v>
       </c>
       <c r="G163" t="s">
         <v>41</v>
       </c>
       <c r="H163" t="s">
-        <v>385</v>
+        <v>383</v>
       </c>
       <c r="I163" t="s">
-        <v>444</v>
+        <v>437</v>
       </c>
       <c r="J163" t="s">
-        <v>439</v>
+        <v>78</v>
       </c>
       <c r="K163" t="s">
-        <v>119</v>
+        <v>78</v>
       </c>
       <c r="L163" t="s">
-        <v>34</v>
+        <v>411</v>
       </c>
       <c r="M163" t="s">
         <v>382</v>
@@ -11767,10 +11767,10 @@
         <v>47</v>
       </c>
       <c r="O163" t="s">
-        <v>269</v>
+        <v>169</v>
       </c>
       <c r="P163" t="s">
-        <v>444</v>
+        <v>437</v>
       </c>
       <c r="Q163" t="s">
         <v>47</v>
@@ -11793,28 +11793,28 @@
         <v>34</v>
       </c>
       <c r="E164" t="s">
-        <v>445</v>
+        <v>438</v>
       </c>
       <c r="F164" t="s">
-        <v>208</v>
+        <v>247</v>
       </c>
       <c r="G164" t="s">
         <v>41</v>
       </c>
       <c r="H164" t="s">
-        <v>389</v>
+        <v>383</v>
       </c>
       <c r="I164" t="s">
-        <v>446</v>
+        <v>439</v>
       </c>
       <c r="J164" t="s">
-        <v>447</v>
+        <v>73</v>
       </c>
       <c r="K164" t="s">
-        <v>119</v>
+        <v>73</v>
       </c>
       <c r="L164" t="s">
-        <v>34</v>
+        <v>411</v>
       </c>
       <c r="M164" t="s">
         <v>382</v>
@@ -11823,10 +11823,10 @@
         <v>47</v>
       </c>
       <c r="O164" t="s">
-        <v>269</v>
+        <v>385</v>
       </c>
       <c r="P164" t="s">
-        <v>446</v>
+        <v>439</v>
       </c>
       <c r="Q164" t="s">
         <v>47</v>
@@ -11849,28 +11849,28 @@
         <v>34</v>
       </c>
       <c r="E165" t="s">
-        <v>448</v>
+        <v>303</v>
       </c>
       <c r="F165" t="s">
-        <v>208</v>
+        <v>247</v>
       </c>
       <c r="G165" t="s">
         <v>41</v>
       </c>
       <c r="H165" t="s">
-        <v>389</v>
+        <v>383</v>
       </c>
       <c r="I165" t="s">
-        <v>449</v>
+        <v>440</v>
       </c>
       <c r="J165" t="s">
-        <v>447</v>
+        <v>119</v>
       </c>
       <c r="K165" t="s">
-        <v>97</v>
+        <v>119</v>
       </c>
       <c r="L165" t="s">
-        <v>34</v>
+        <v>411</v>
       </c>
       <c r="M165" t="s">
         <v>382</v>
@@ -11879,10 +11879,10 @@
         <v>47</v>
       </c>
       <c r="O165" t="s">
-        <v>98</v>
+        <v>149</v>
       </c>
       <c r="P165" t="s">
-        <v>449</v>
+        <v>440</v>
       </c>
       <c r="Q165" t="s">
         <v>47</v>
@@ -11905,28 +11905,28 @@
         <v>34</v>
       </c>
       <c r="E166" t="s">
-        <v>87</v>
+        <v>298</v>
       </c>
       <c r="F166" t="s">
-        <v>208</v>
+        <v>247</v>
       </c>
       <c r="G166" t="s">
         <v>41</v>
       </c>
       <c r="H166" t="s">
-        <v>389</v>
+        <v>383</v>
       </c>
       <c r="I166" t="s">
-        <v>450</v>
+        <v>441</v>
       </c>
       <c r="J166" t="s">
-        <v>447</v>
+        <v>73</v>
       </c>
       <c r="K166" t="s">
         <v>73</v>
       </c>
       <c r="L166" t="s">
-        <v>34</v>
+        <v>411</v>
       </c>
       <c r="M166" t="s">
         <v>382</v>
@@ -11935,10 +11935,10 @@
         <v>47</v>
       </c>
       <c r="O166" t="s">
-        <v>412</v>
+        <v>115</v>
       </c>
       <c r="P166" t="s">
-        <v>450</v>
+        <v>441</v>
       </c>
       <c r="Q166" t="s">
         <v>47</v>
@@ -11961,28 +11961,28 @@
         <v>34</v>
       </c>
       <c r="E167" t="s">
-        <v>166</v>
+        <v>442</v>
       </c>
       <c r="F167" t="s">
-        <v>208</v>
+        <v>247</v>
       </c>
       <c r="G167" t="s">
         <v>41</v>
       </c>
       <c r="H167" t="s">
-        <v>385</v>
+        <v>388</v>
       </c>
       <c r="I167" t="s">
-        <v>451</v>
+        <v>443</v>
       </c>
       <c r="J167" t="s">
-        <v>78</v>
+        <v>133</v>
       </c>
       <c r="K167" t="s">
-        <v>78</v>
+        <v>133</v>
       </c>
       <c r="L167" t="s">
-        <v>34</v>
+        <v>411</v>
       </c>
       <c r="M167" t="s">
         <v>382</v>
@@ -11991,10 +11991,10 @@
         <v>47</v>
       </c>
       <c r="O167" t="s">
-        <v>169</v>
+        <v>145</v>
       </c>
       <c r="P167" t="s">
-        <v>451</v>
+        <v>443</v>
       </c>
       <c r="Q167" t="s">
         <v>47</v>
@@ -12017,28 +12017,28 @@
         <v>34</v>
       </c>
       <c r="E168" t="s">
-        <v>452</v>
+        <v>444</v>
       </c>
       <c r="F168" t="s">
-        <v>208</v>
+        <v>247</v>
       </c>
       <c r="G168" t="s">
         <v>41</v>
       </c>
       <c r="H168" t="s">
-        <v>385</v>
+        <v>388</v>
       </c>
       <c r="I168" t="s">
-        <v>453</v>
+        <v>445</v>
       </c>
       <c r="J168" t="s">
-        <v>119</v>
+        <v>105</v>
       </c>
       <c r="K168" t="s">
-        <v>119</v>
+        <v>105</v>
       </c>
       <c r="L168" t="s">
-        <v>34</v>
+        <v>411</v>
       </c>
       <c r="M168" t="s">
         <v>382</v>
@@ -12047,10 +12047,10 @@
         <v>47</v>
       </c>
       <c r="O168" t="s">
-        <v>269</v>
+        <v>112</v>
       </c>
       <c r="P168" t="s">
-        <v>453</v>
+        <v>445</v>
       </c>
       <c r="Q168" t="s">
         <v>47</v>
@@ -12073,28 +12073,28 @@
         <v>34</v>
       </c>
       <c r="E169" t="s">
-        <v>454</v>
+        <v>446</v>
       </c>
       <c r="F169" t="s">
-        <v>208</v>
+        <v>247</v>
       </c>
       <c r="G169" t="s">
         <v>41</v>
       </c>
       <c r="H169" t="s">
-        <v>385</v>
+        <v>383</v>
       </c>
       <c r="I169" t="s">
-        <v>455</v>
+        <v>447</v>
       </c>
       <c r="J169" t="s">
-        <v>68</v>
+        <v>120</v>
       </c>
       <c r="K169" t="s">
-        <v>68</v>
+        <v>120</v>
       </c>
       <c r="L169" t="s">
-        <v>34</v>
+        <v>411</v>
       </c>
       <c r="M169" t="s">
         <v>382</v>
@@ -12103,10 +12103,10 @@
         <v>47</v>
       </c>
       <c r="O169" t="s">
-        <v>262</v>
+        <v>152</v>
       </c>
       <c r="P169" t="s">
-        <v>455</v>
+        <v>447</v>
       </c>
       <c r="Q169" t="s">
         <v>47</v>
@@ -12129,19 +12129,19 @@
         <v>34</v>
       </c>
       <c r="E170" t="s">
-        <v>87</v>
+        <v>448</v>
       </c>
       <c r="F170" t="s">
-        <v>208</v>
+        <v>247</v>
       </c>
       <c r="G170" t="s">
         <v>41</v>
       </c>
       <c r="H170" t="s">
-        <v>385</v>
+        <v>383</v>
       </c>
       <c r="I170" t="s">
-        <v>456</v>
+        <v>449</v>
       </c>
       <c r="J170" t="s">
         <v>73</v>
@@ -12150,7 +12150,7 @@
         <v>73</v>
       </c>
       <c r="L170" t="s">
-        <v>34</v>
+        <v>411</v>
       </c>
       <c r="M170" t="s">
         <v>382</v>
@@ -12159,10 +12159,10 @@
         <v>47</v>
       </c>
       <c r="O170" t="s">
-        <v>412</v>
+        <v>294</v>
       </c>
       <c r="P170" t="s">
-        <v>456</v>
+        <v>449</v>
       </c>
       <c r="Q170" t="s">
         <v>47</v>
@@ -12185,28 +12185,28 @@
         <v>34</v>
       </c>
       <c r="E171" t="s">
-        <v>457</v>
+        <v>280</v>
       </c>
       <c r="F171" t="s">
-        <v>208</v>
+        <v>247</v>
       </c>
       <c r="G171" t="s">
         <v>41</v>
       </c>
       <c r="H171" t="s">
-        <v>385</v>
+        <v>383</v>
       </c>
       <c r="I171" t="s">
-        <v>458</v>
+        <v>450</v>
       </c>
       <c r="J171" t="s">
-        <v>97</v>
+        <v>133</v>
       </c>
       <c r="K171" t="s">
-        <v>97</v>
+        <v>133</v>
       </c>
       <c r="L171" t="s">
-        <v>34</v>
+        <v>411</v>
       </c>
       <c r="M171" t="s">
         <v>382</v>
@@ -12215,10 +12215,10 @@
         <v>47</v>
       </c>
       <c r="O171" t="s">
-        <v>98</v>
+        <v>145</v>
       </c>
       <c r="P171" t="s">
-        <v>458</v>
+        <v>450</v>
       </c>
       <c r="Q171" t="s">
         <v>47</v>
@@ -12241,28 +12241,28 @@
         <v>34</v>
       </c>
       <c r="E172" t="s">
-        <v>113</v>
+        <v>451</v>
       </c>
       <c r="F172" t="s">
-        <v>208</v>
+        <v>247</v>
       </c>
       <c r="G172" t="s">
         <v>41</v>
       </c>
       <c r="H172" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
       <c r="I172" t="s">
-        <v>459</v>
+        <v>452</v>
       </c>
       <c r="J172" t="s">
-        <v>73</v>
+        <v>120</v>
       </c>
       <c r="K172" t="s">
-        <v>73</v>
+        <v>120</v>
       </c>
       <c r="L172" t="s">
-        <v>34</v>
+        <v>411</v>
       </c>
       <c r="M172" t="s">
         <v>382</v>
@@ -12271,10 +12271,10 @@
         <v>47</v>
       </c>
       <c r="O172" t="s">
-        <v>115</v>
+        <v>152</v>
       </c>
       <c r="P172" t="s">
-        <v>459</v>
+        <v>452</v>
       </c>
       <c r="Q172" t="s">
         <v>47</v>
@@ -12297,19 +12297,19 @@
         <v>34</v>
       </c>
       <c r="E173" t="s">
-        <v>113</v>
+        <v>453</v>
       </c>
       <c r="F173" t="s">
-        <v>208</v>
+        <v>247</v>
       </c>
       <c r="G173" t="s">
         <v>41</v>
       </c>
       <c r="H173" t="s">
-        <v>385</v>
+        <v>388</v>
       </c>
       <c r="I173" t="s">
-        <v>460</v>
+        <v>454</v>
       </c>
       <c r="J173" t="s">
         <v>73</v>
@@ -12318,7 +12318,7 @@
         <v>73</v>
       </c>
       <c r="L173" t="s">
-        <v>34</v>
+        <v>411</v>
       </c>
       <c r="M173" t="s">
         <v>382</v>
@@ -12327,10 +12327,10 @@
         <v>47</v>
       </c>
       <c r="O173" t="s">
-        <v>115</v>
+        <v>294</v>
       </c>
       <c r="P173" t="s">
-        <v>460</v>
+        <v>454</v>
       </c>
       <c r="Q173" t="s">
         <v>47</v>
@@ -12353,7 +12353,7 @@
         <v>34</v>
       </c>
       <c r="E174" t="s">
-        <v>461</v>
+        <v>455</v>
       </c>
       <c r="F174" t="s">
         <v>208</v>
@@ -12362,16 +12362,16 @@
         <v>41</v>
       </c>
       <c r="H174" t="s">
-        <v>385</v>
+        <v>388</v>
       </c>
       <c r="I174" t="s">
-        <v>462</v>
+        <v>456</v>
       </c>
       <c r="J174" t="s">
-        <v>68</v>
+        <v>45</v>
       </c>
       <c r="K174" t="s">
-        <v>68</v>
+        <v>45</v>
       </c>
       <c r="L174" t="s">
         <v>34</v>
@@ -12383,10 +12383,10 @@
         <v>47</v>
       </c>
       <c r="O174" t="s">
-        <v>262</v>
+        <v>48</v>
       </c>
       <c r="P174" t="s">
-        <v>462</v>
+        <v>456</v>
       </c>
       <c r="Q174" t="s">
         <v>47</v>
@@ -12409,7 +12409,7 @@
         <v>34</v>
       </c>
       <c r="E175" t="s">
-        <v>445</v>
+        <v>457</v>
       </c>
       <c r="F175" t="s">
         <v>208</v>
@@ -12418,16 +12418,16 @@
         <v>41</v>
       </c>
       <c r="H175" t="s">
-        <v>385</v>
+        <v>388</v>
       </c>
       <c r="I175" t="s">
-        <v>463</v>
+        <v>458</v>
       </c>
       <c r="J175" t="s">
-        <v>119</v>
+        <v>45</v>
       </c>
       <c r="K175" t="s">
-        <v>119</v>
+        <v>45</v>
       </c>
       <c r="L175" t="s">
         <v>34</v>
@@ -12439,10 +12439,10 @@
         <v>47</v>
       </c>
       <c r="O175" t="s">
-        <v>269</v>
+        <v>459</v>
       </c>
       <c r="P175" t="s">
-        <v>463</v>
+        <v>458</v>
       </c>
       <c r="Q175" t="s">
         <v>47</v>
@@ -12465,7 +12465,7 @@
         <v>34</v>
       </c>
       <c r="E176" t="s">
-        <v>464</v>
+        <v>94</v>
       </c>
       <c r="F176" t="s">
         <v>208</v>
@@ -12474,16 +12474,16 @@
         <v>41</v>
       </c>
       <c r="H176" t="s">
-        <v>385</v>
+        <v>383</v>
       </c>
       <c r="I176" t="s">
-        <v>463</v>
+        <v>460</v>
       </c>
       <c r="J176" t="s">
-        <v>78</v>
+        <v>461</v>
       </c>
       <c r="K176" t="s">
-        <v>78</v>
+        <v>97</v>
       </c>
       <c r="L176" t="s">
         <v>34</v>
@@ -12495,10 +12495,10 @@
         <v>47</v>
       </c>
       <c r="O176" t="s">
-        <v>169</v>
+        <v>98</v>
       </c>
       <c r="P176" t="s">
-        <v>463</v>
+        <v>460</v>
       </c>
       <c r="Q176" t="s">
         <v>47</v>
@@ -12521,7 +12521,7 @@
         <v>34</v>
       </c>
       <c r="E177" t="s">
-        <v>465</v>
+        <v>462</v>
       </c>
       <c r="F177" t="s">
         <v>208</v>
@@ -12530,16 +12530,16 @@
         <v>41</v>
       </c>
       <c r="H177" t="s">
-        <v>385</v>
+        <v>388</v>
       </c>
       <c r="I177" t="s">
         <v>463</v>
       </c>
       <c r="J177" t="s">
-        <v>68</v>
+        <v>464</v>
       </c>
       <c r="K177" t="s">
-        <v>68</v>
+        <v>119</v>
       </c>
       <c r="L177" t="s">
         <v>34</v>
@@ -12551,7 +12551,7 @@
         <v>47</v>
       </c>
       <c r="O177" t="s">
-        <v>262</v>
+        <v>269</v>
       </c>
       <c r="P177" t="s">
         <v>463</v>
@@ -12577,7 +12577,7 @@
         <v>34</v>
       </c>
       <c r="E178" t="s">
-        <v>466</v>
+        <v>94</v>
       </c>
       <c r="F178" t="s">
         <v>208</v>
@@ -12586,16 +12586,16 @@
         <v>41</v>
       </c>
       <c r="H178" t="s">
-        <v>385</v>
+        <v>388</v>
       </c>
       <c r="I178" t="s">
-        <v>467</v>
+        <v>465</v>
       </c>
       <c r="J178" t="s">
-        <v>73</v>
+        <v>97</v>
       </c>
       <c r="K178" t="s">
-        <v>73</v>
+        <v>97</v>
       </c>
       <c r="L178" t="s">
         <v>34</v>
@@ -12607,10 +12607,10 @@
         <v>47</v>
       </c>
       <c r="O178" t="s">
-        <v>115</v>
+        <v>98</v>
       </c>
       <c r="P178" t="s">
-        <v>467</v>
+        <v>465</v>
       </c>
       <c r="Q178" t="s">
         <v>47</v>
@@ -12633,7 +12633,7 @@
         <v>34</v>
       </c>
       <c r="E179" t="s">
-        <v>150</v>
+        <v>462</v>
       </c>
       <c r="F179" t="s">
         <v>208</v>
@@ -12642,16 +12642,16 @@
         <v>41</v>
       </c>
       <c r="H179" t="s">
-        <v>389</v>
+        <v>383</v>
       </c>
       <c r="I179" t="s">
-        <v>450</v>
+        <v>466</v>
       </c>
       <c r="J179" t="s">
-        <v>120</v>
+        <v>461</v>
       </c>
       <c r="K179" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="L179" t="s">
         <v>34</v>
@@ -12663,10 +12663,10 @@
         <v>47</v>
       </c>
       <c r="O179" t="s">
-        <v>152</v>
+        <v>269</v>
       </c>
       <c r="P179" t="s">
-        <v>450</v>
+        <v>466</v>
       </c>
       <c r="Q179" t="s">
         <v>47</v>
@@ -12689,7 +12689,7 @@
         <v>34</v>
       </c>
       <c r="E180" t="s">
-        <v>110</v>
+        <v>393</v>
       </c>
       <c r="F180" t="s">
         <v>208</v>
@@ -12698,16 +12698,16 @@
         <v>41</v>
       </c>
       <c r="H180" t="s">
-        <v>385</v>
+        <v>388</v>
       </c>
       <c r="I180" t="s">
+        <v>467</v>
+      </c>
+      <c r="J180" t="s">
         <v>468</v>
       </c>
-      <c r="J180" t="s">
-        <v>105</v>
-      </c>
       <c r="K180" t="s">
-        <v>105</v>
+        <v>119</v>
       </c>
       <c r="L180" t="s">
         <v>34</v>
@@ -12719,10 +12719,10 @@
         <v>47</v>
       </c>
       <c r="O180" t="s">
-        <v>112</v>
+        <v>269</v>
       </c>
       <c r="P180" t="s">
-        <v>468</v>
+        <v>467</v>
       </c>
       <c r="Q180" t="s">
         <v>47</v>
@@ -12754,16 +12754,16 @@
         <v>41</v>
       </c>
       <c r="H181" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
       <c r="I181" t="s">
         <v>470</v>
       </c>
       <c r="J181" t="s">
-        <v>73</v>
+        <v>468</v>
       </c>
       <c r="K181" t="s">
-        <v>73</v>
+        <v>97</v>
       </c>
       <c r="L181" t="s">
         <v>34</v>
@@ -12775,7 +12775,7 @@
         <v>47</v>
       </c>
       <c r="O181" t="s">
-        <v>115</v>
+        <v>98</v>
       </c>
       <c r="P181" t="s">
         <v>470</v>
@@ -12801,7 +12801,7 @@
         <v>34</v>
       </c>
       <c r="E182" t="s">
-        <v>150</v>
+        <v>87</v>
       </c>
       <c r="F182" t="s">
         <v>208</v>
@@ -12810,16 +12810,16 @@
         <v>41</v>
       </c>
       <c r="H182" t="s">
-        <v>385</v>
+        <v>388</v>
       </c>
       <c r="I182" t="s">
-        <v>463</v>
+        <v>399</v>
       </c>
       <c r="J182" t="s">
-        <v>120</v>
+        <v>468</v>
       </c>
       <c r="K182" t="s">
-        <v>120</v>
+        <v>73</v>
       </c>
       <c r="L182" t="s">
         <v>34</v>
@@ -12831,10 +12831,10 @@
         <v>47</v>
       </c>
       <c r="O182" t="s">
-        <v>152</v>
+        <v>385</v>
       </c>
       <c r="P182" t="s">
-        <v>463</v>
+        <v>399</v>
       </c>
       <c r="Q182" t="s">
         <v>47</v>
@@ -12857,7 +12857,7 @@
         <v>34</v>
       </c>
       <c r="E183" t="s">
-        <v>471</v>
+        <v>166</v>
       </c>
       <c r="F183" t="s">
         <v>208</v>
@@ -12866,16 +12866,16 @@
         <v>41</v>
       </c>
       <c r="H183" t="s">
-        <v>385</v>
+        <v>383</v>
       </c>
       <c r="I183" t="s">
-        <v>472</v>
+        <v>471</v>
       </c>
       <c r="J183" t="s">
-        <v>73</v>
+        <v>78</v>
       </c>
       <c r="K183" t="s">
-        <v>73</v>
+        <v>78</v>
       </c>
       <c r="L183" t="s">
         <v>34</v>
@@ -12887,10 +12887,10 @@
         <v>47</v>
       </c>
       <c r="O183" t="s">
-        <v>115</v>
+        <v>169</v>
       </c>
       <c r="P183" t="s">
-        <v>472</v>
+        <v>471</v>
       </c>
       <c r="Q183" t="s">
         <v>47</v>
@@ -12913,7 +12913,7 @@
         <v>34</v>
       </c>
       <c r="E184" t="s">
-        <v>473</v>
+        <v>472</v>
       </c>
       <c r="F184" t="s">
         <v>208</v>
@@ -12922,16 +12922,16 @@
         <v>41</v>
       </c>
       <c r="H184" t="s">
-        <v>385</v>
+        <v>383</v>
       </c>
       <c r="I184" t="s">
-        <v>474</v>
+        <v>473</v>
       </c>
       <c r="J184" t="s">
-        <v>73</v>
+        <v>119</v>
       </c>
       <c r="K184" t="s">
-        <v>73</v>
+        <v>119</v>
       </c>
       <c r="L184" t="s">
         <v>34</v>
@@ -12943,10 +12943,10 @@
         <v>47</v>
       </c>
       <c r="O184" t="s">
-        <v>294</v>
+        <v>269</v>
       </c>
       <c r="P184" t="s">
-        <v>474</v>
+        <v>473</v>
       </c>
       <c r="Q184" t="s">
         <v>47</v>
@@ -12969,7 +12969,7 @@
         <v>34</v>
       </c>
       <c r="E185" t="s">
-        <v>473</v>
+        <v>474</v>
       </c>
       <c r="F185" t="s">
         <v>208</v>
@@ -12978,16 +12978,16 @@
         <v>41</v>
       </c>
       <c r="H185" t="s">
-        <v>389</v>
+        <v>383</v>
       </c>
       <c r="I185" t="s">
         <v>475</v>
       </c>
       <c r="J185" t="s">
-        <v>73</v>
+        <v>68</v>
       </c>
       <c r="K185" t="s">
-        <v>73</v>
+        <v>68</v>
       </c>
       <c r="L185" t="s">
         <v>34</v>
@@ -12999,7 +12999,7 @@
         <v>47</v>
       </c>
       <c r="O185" t="s">
-        <v>294</v>
+        <v>262</v>
       </c>
       <c r="P185" t="s">
         <v>475</v>
@@ -18039,7 +18039,7 @@
         <v>47</v>
       </c>
       <c r="O275" t="s">
-        <v>412</v>
+        <v>385</v>
       </c>
       <c r="P275" t="s">
         <v>500</v>
@@ -18242,7 +18242,7 @@
         <v>41</v>
       </c>
       <c r="H279" t="s">
-        <v>197</v>
+        <v>192</v>
       </c>
       <c r="I279" t="s">
         <v>581</v>
@@ -18289,7 +18289,7 @@
         <v>34</v>
       </c>
       <c r="E280" t="s">
-        <v>391</v>
+        <v>414</v>
       </c>
       <c r="F280" t="s">
         <v>484</v>
@@ -18298,7 +18298,7 @@
         <v>41</v>
       </c>
       <c r="H280" t="s">
-        <v>197</v>
+        <v>192</v>
       </c>
       <c r="I280" t="s">
         <v>494</v>
@@ -18354,7 +18354,7 @@
         <v>41</v>
       </c>
       <c r="H281" t="s">
-        <v>197</v>
+        <v>192</v>
       </c>
       <c r="I281" t="s">
         <v>550</v>
@@ -18410,7 +18410,7 @@
         <v>41</v>
       </c>
       <c r="H282" t="s">
-        <v>197</v>
+        <v>192</v>
       </c>
       <c r="I282" t="s">
         <v>489</v>
@@ -18522,7 +18522,7 @@
         <v>41</v>
       </c>
       <c r="H284" t="s">
-        <v>197</v>
+        <v>192</v>
       </c>
       <c r="I284" t="s">
         <v>585</v>
@@ -18578,7 +18578,7 @@
         <v>41</v>
       </c>
       <c r="H285" t="s">
-        <v>197</v>
+        <v>192</v>
       </c>
       <c r="I285" t="s">
         <v>588</v>
@@ -18634,7 +18634,7 @@
         <v>41</v>
       </c>
       <c r="H286" t="s">
-        <v>197</v>
+        <v>192</v>
       </c>
       <c r="I286" t="s">
         <v>589</v>
@@ -18690,7 +18690,7 @@
         <v>41</v>
       </c>
       <c r="H287" t="s">
-        <v>197</v>
+        <v>192</v>
       </c>
       <c r="I287" t="s">
         <v>590</v>
@@ -18746,7 +18746,7 @@
         <v>41</v>
       </c>
       <c r="H288" t="s">
-        <v>197</v>
+        <v>192</v>
       </c>
       <c r="I288" t="s">
         <v>591</v>
@@ -18849,7 +18849,7 @@
         <v>34</v>
       </c>
       <c r="E290" t="s">
-        <v>473</v>
+        <v>405</v>
       </c>
       <c r="F290" t="s">
         <v>208</v>
@@ -19129,7 +19129,7 @@
         <v>34</v>
       </c>
       <c r="E295" t="s">
-        <v>454</v>
+        <v>474</v>
       </c>
       <c r="F295" t="s">
         <v>208</v>
@@ -19185,7 +19185,7 @@
         <v>34</v>
       </c>
       <c r="E296" t="s">
-        <v>440</v>
+        <v>462</v>
       </c>
       <c r="F296" t="s">
         <v>208</v>
@@ -19418,7 +19418,7 @@
         <v>41</v>
       </c>
       <c r="H300" t="s">
-        <v>197</v>
+        <v>192</v>
       </c>
       <c r="I300" t="s">
         <v>612</v>
@@ -20261,7 +20261,7 @@
         <v>638</v>
       </c>
       <c r="I315" t="s">
-        <v>455</v>
+        <v>475</v>
       </c>
       <c r="J315" t="s">
         <v>105</v>
@@ -20282,7 +20282,7 @@
         <v>112</v>
       </c>
       <c r="P315" t="s">
-        <v>455</v>
+        <v>475</v>
       </c>
       <c r="Q315" t="s">
         <v>47</v>
@@ -20305,7 +20305,7 @@
         <v>34</v>
       </c>
       <c r="E316" t="s">
-        <v>473</v>
+        <v>405</v>
       </c>
       <c r="F316" t="s">
         <v>208</v>
@@ -20417,7 +20417,7 @@
         <v>34</v>
       </c>
       <c r="E318" t="s">
-        <v>454</v>
+        <v>474</v>
       </c>
       <c r="F318" t="s">
         <v>208</v>
@@ -20977,7 +20977,7 @@
         <v>34</v>
       </c>
       <c r="E328" t="s">
-        <v>440</v>
+        <v>462</v>
       </c>
       <c r="F328" t="s">
         <v>208</v>
@@ -21985,7 +21985,7 @@
         <v>33</v>
       </c>
       <c r="E346" t="s">
-        <v>272</v>
+        <v>263</v>
       </c>
       <c r="F346" t="s">
         <v>40</v>
@@ -22000,10 +22000,10 @@
         <v>92</v>
       </c>
       <c r="J346" t="s">
-        <v>133</v>
+        <v>119</v>
       </c>
       <c r="K346" t="s">
-        <v>133</v>
+        <v>119</v>
       </c>
       <c r="L346" t="s">
         <v>34</v>
@@ -22015,7 +22015,7 @@
         <v>47</v>
       </c>
       <c r="O346" t="s">
-        <v>145</v>
+        <v>149</v>
       </c>
       <c r="P346" t="s">
         <v>92</v>
@@ -22041,7 +22041,7 @@
         <v>34</v>
       </c>
       <c r="E347" t="s">
-        <v>290</v>
+        <v>258</v>
       </c>
       <c r="F347" t="s">
         <v>40</v>
@@ -22071,7 +22071,7 @@
         <v>47</v>
       </c>
       <c r="O347" t="s">
-        <v>294</v>
+        <v>115</v>
       </c>
       <c r="P347" t="s">
         <v>92</v>
@@ -22153,10 +22153,10 @@
         <v>34</v>
       </c>
       <c r="E349" t="s">
-        <v>250</v>
+        <v>531</v>
       </c>
       <c r="F349" t="s">
-        <v>40</v>
+        <v>709</v>
       </c>
       <c r="G349" t="s">
         <v>41</v>
@@ -22168,10 +22168,10 @@
         <v>92</v>
       </c>
       <c r="J349" t="s">
-        <v>105</v>
+        <v>124</v>
       </c>
       <c r="K349" t="s">
-        <v>105</v>
+        <v>124</v>
       </c>
       <c r="L349" t="s">
         <v>34</v>
@@ -22183,13 +22183,13 @@
         <v>47</v>
       </c>
       <c r="O349" t="s">
-        <v>112</v>
+        <v>34</v>
       </c>
       <c r="P349" t="s">
-        <v>92</v>
+        <v>34</v>
       </c>
       <c r="Q349" t="s">
-        <v>47</v>
+        <v>34</v>
       </c>
       <c r="R349" t="s">
         <v>34</v>
@@ -22209,7 +22209,7 @@
         <v>34</v>
       </c>
       <c r="E350" t="s">
-        <v>274</v>
+        <v>290</v>
       </c>
       <c r="F350" t="s">
         <v>40</v>
@@ -22224,10 +22224,10 @@
         <v>92</v>
       </c>
       <c r="J350" t="s">
-        <v>78</v>
+        <v>83</v>
       </c>
       <c r="K350" t="s">
-        <v>78</v>
+        <v>73</v>
       </c>
       <c r="L350" t="s">
         <v>34</v>
@@ -22239,7 +22239,7 @@
         <v>47</v>
       </c>
       <c r="O350" t="s">
-        <v>169</v>
+        <v>294</v>
       </c>
       <c r="P350" t="s">
         <v>92</v>
@@ -22265,7 +22265,7 @@
         <v>34</v>
       </c>
       <c r="E351" t="s">
-        <v>263</v>
+        <v>256</v>
       </c>
       <c r="F351" t="s">
         <v>40</v>
@@ -22280,10 +22280,10 @@
         <v>92</v>
       </c>
       <c r="J351" t="s">
-        <v>119</v>
+        <v>83</v>
       </c>
       <c r="K351" t="s">
-        <v>119</v>
+        <v>73</v>
       </c>
       <c r="L351" t="s">
         <v>34</v>
@@ -22295,7 +22295,7 @@
         <v>47</v>
       </c>
       <c r="O351" t="s">
-        <v>149</v>
+        <v>88</v>
       </c>
       <c r="P351" t="s">
         <v>92</v>
@@ -22321,7 +22321,7 @@
         <v>34</v>
       </c>
       <c r="E352" t="s">
-        <v>256</v>
+        <v>267</v>
       </c>
       <c r="F352" t="s">
         <v>40</v>
@@ -22336,10 +22336,10 @@
         <v>92</v>
       </c>
       <c r="J352" t="s">
-        <v>83</v>
+        <v>119</v>
       </c>
       <c r="K352" t="s">
-        <v>73</v>
+        <v>119</v>
       </c>
       <c r="L352" t="s">
         <v>34</v>
@@ -22351,7 +22351,7 @@
         <v>47</v>
       </c>
       <c r="O352" t="s">
-        <v>88</v>
+        <v>269</v>
       </c>
       <c r="P352" t="s">
         <v>92</v>
@@ -22433,7 +22433,7 @@
         <v>34</v>
       </c>
       <c r="E354" t="s">
-        <v>258</v>
+        <v>274</v>
       </c>
       <c r="F354" t="s">
         <v>40</v>
@@ -22448,10 +22448,10 @@
         <v>92</v>
       </c>
       <c r="J354" t="s">
-        <v>83</v>
+        <v>78</v>
       </c>
       <c r="K354" t="s">
-        <v>73</v>
+        <v>78</v>
       </c>
       <c r="L354" t="s">
         <v>34</v>
@@ -22463,7 +22463,7 @@
         <v>47</v>
       </c>
       <c r="O354" t="s">
-        <v>115</v>
+        <v>169</v>
       </c>
       <c r="P354" t="s">
         <v>92</v>
@@ -22489,10 +22489,10 @@
         <v>34</v>
       </c>
       <c r="E355" t="s">
-        <v>531</v>
+        <v>272</v>
       </c>
       <c r="F355" t="s">
-        <v>709</v>
+        <v>40</v>
       </c>
       <c r="G355" t="s">
         <v>41</v>
@@ -22504,10 +22504,10 @@
         <v>92</v>
       </c>
       <c r="J355" t="s">
-        <v>124</v>
+        <v>133</v>
       </c>
       <c r="K355" t="s">
-        <v>124</v>
+        <v>133</v>
       </c>
       <c r="L355" t="s">
         <v>34</v>
@@ -22519,13 +22519,13 @@
         <v>47</v>
       </c>
       <c r="O355" t="s">
-        <v>34</v>
+        <v>145</v>
       </c>
       <c r="P355" t="s">
-        <v>34</v>
+        <v>92</v>
       </c>
       <c r="Q355" t="s">
-        <v>34</v>
+        <v>47</v>
       </c>
       <c r="R355" t="s">
         <v>34</v>
@@ -22545,7 +22545,7 @@
         <v>34</v>
       </c>
       <c r="E356" t="s">
-        <v>254</v>
+        <v>250</v>
       </c>
       <c r="F356" t="s">
         <v>40</v>
@@ -22560,10 +22560,10 @@
         <v>92</v>
       </c>
       <c r="J356" t="s">
-        <v>97</v>
+        <v>105</v>
       </c>
       <c r="K356" t="s">
-        <v>97</v>
+        <v>105</v>
       </c>
       <c r="L356" t="s">
         <v>34</v>
@@ -22575,7 +22575,7 @@
         <v>47</v>
       </c>
       <c r="O356" t="s">
-        <v>98</v>
+        <v>112</v>
       </c>
       <c r="P356" t="s">
         <v>92</v>
@@ -22657,7 +22657,7 @@
         <v>34</v>
       </c>
       <c r="E358" t="s">
-        <v>260</v>
+        <v>487</v>
       </c>
       <c r="F358" t="s">
         <v>40</v>
@@ -22672,10 +22672,10 @@
         <v>92</v>
       </c>
       <c r="J358" t="s">
-        <v>83</v>
+        <v>78</v>
       </c>
       <c r="K358" t="s">
-        <v>68</v>
+        <v>78</v>
       </c>
       <c r="L358" t="s">
         <v>34</v>
@@ -22687,7 +22687,7 @@
         <v>47</v>
       </c>
       <c r="O358" t="s">
-        <v>262</v>
+        <v>79</v>
       </c>
       <c r="P358" t="s">
         <v>92</v>
@@ -22713,7 +22713,7 @@
         <v>34</v>
       </c>
       <c r="E359" t="s">
-        <v>267</v>
+        <v>254</v>
       </c>
       <c r="F359" t="s">
         <v>40</v>
@@ -22728,10 +22728,10 @@
         <v>92</v>
       </c>
       <c r="J359" t="s">
-        <v>119</v>
+        <v>97</v>
       </c>
       <c r="K359" t="s">
-        <v>119</v>
+        <v>97</v>
       </c>
       <c r="L359" t="s">
         <v>34</v>
@@ -22743,7 +22743,7 @@
         <v>47</v>
       </c>
       <c r="O359" t="s">
-        <v>269</v>
+        <v>98</v>
       </c>
       <c r="P359" t="s">
         <v>92</v>
@@ -22769,7 +22769,7 @@
         <v>34</v>
       </c>
       <c r="E360" t="s">
-        <v>487</v>
+        <v>260</v>
       </c>
       <c r="F360" t="s">
         <v>40</v>
@@ -22784,10 +22784,10 @@
         <v>92</v>
       </c>
       <c r="J360" t="s">
-        <v>78</v>
+        <v>83</v>
       </c>
       <c r="K360" t="s">
-        <v>78</v>
+        <v>68</v>
       </c>
       <c r="L360" t="s">
         <v>34</v>
@@ -22799,7 +22799,7 @@
         <v>47</v>
       </c>
       <c r="O360" t="s">
-        <v>79</v>
+        <v>262</v>
       </c>
       <c r="P360" t="s">
         <v>92</v>
@@ -22937,7 +22937,7 @@
         <v>33</v>
       </c>
       <c r="E363" t="s">
-        <v>720</v>
+        <v>227</v>
       </c>
       <c r="F363" t="s">
         <v>40</v>
@@ -22946,16 +22946,16 @@
         <v>41</v>
       </c>
       <c r="H363" t="s">
+        <v>720</v>
+      </c>
+      <c r="I363" t="s">
         <v>721</v>
       </c>
-      <c r="I363" t="s">
+      <c r="J363" t="s">
         <v>722</v>
       </c>
-      <c r="J363" t="s">
-        <v>369</v>
-      </c>
       <c r="K363" t="s">
-        <v>45</v>
+        <v>67</v>
       </c>
       <c r="L363" t="s">
         <v>723</v>
@@ -22970,7 +22970,7 @@
         <v>48</v>
       </c>
       <c r="P363" t="s">
-        <v>722</v>
+        <v>721</v>
       </c>
       <c r="Q363" t="s">
         <v>47</v>
@@ -22993,7 +22993,7 @@
         <v>34</v>
       </c>
       <c r="E364" t="s">
-        <v>720</v>
+        <v>724</v>
       </c>
       <c r="F364" t="s">
         <v>40</v>
@@ -23002,19 +23002,19 @@
         <v>41</v>
       </c>
       <c r="H364" t="s">
-        <v>724</v>
+        <v>725</v>
       </c>
       <c r="I364" t="s">
-        <v>725</v>
+        <v>726</v>
       </c>
       <c r="J364" t="s">
-        <v>726</v>
+        <v>727</v>
       </c>
       <c r="K364" t="s">
-        <v>727</v>
+        <v>728</v>
       </c>
       <c r="L364" t="s">
-        <v>728</v>
+        <v>729</v>
       </c>
       <c r="M364" t="s">
         <v>718</v>
@@ -23026,7 +23026,7 @@
         <v>48</v>
       </c>
       <c r="P364" t="s">
-        <v>725</v>
+        <v>726</v>
       </c>
       <c r="Q364" t="s">
         <v>47</v>
@@ -23049,7 +23049,7 @@
         <v>34</v>
       </c>
       <c r="E365" t="s">
-        <v>729</v>
+        <v>724</v>
       </c>
       <c r="F365" t="s">
         <v>40</v>
@@ -23064,13 +23064,13 @@
         <v>731</v>
       </c>
       <c r="J365" t="s">
-        <v>230</v>
+        <v>369</v>
       </c>
       <c r="K365" t="s">
+        <v>45</v>
+      </c>
+      <c r="L365" t="s">
         <v>732</v>
-      </c>
-      <c r="L365" t="s">
-        <v>733</v>
       </c>
       <c r="M365" t="s">
         <v>718</v>
@@ -23105,7 +23105,7 @@
         <v>34</v>
       </c>
       <c r="E366" t="s">
-        <v>227</v>
+        <v>733</v>
       </c>
       <c r="F366" t="s">
         <v>40</v>
@@ -23120,10 +23120,10 @@
         <v>735</v>
       </c>
       <c r="J366" t="s">
+        <v>230</v>
+      </c>
+      <c r="K366" t="s">
         <v>736</v>
-      </c>
-      <c r="K366" t="s">
-        <v>67</v>
       </c>
       <c r="L366" t="s">
         <v>737</v>
@@ -23385,7 +23385,7 @@
         <v>33</v>
       </c>
       <c r="E371" t="s">
-        <v>720</v>
+        <v>724</v>
       </c>
       <c r="F371" t="s">
         <v>40</v>
@@ -23400,7 +23400,7 @@
         <v>750</v>
       </c>
       <c r="J371" t="s">
-        <v>726</v>
+        <v>727</v>
       </c>
       <c r="K371" t="s">
         <v>45</v>
@@ -23609,7 +23609,7 @@
         <v>34</v>
       </c>
       <c r="E375" t="s">
-        <v>720</v>
+        <v>724</v>
       </c>
       <c r="F375" t="s">
         <v>40</v>
@@ -23624,7 +23624,7 @@
         <v>762</v>
       </c>
       <c r="J375" t="s">
-        <v>726</v>
+        <v>727</v>
       </c>
       <c r="K375" t="s">
         <v>45</v>
@@ -23665,7 +23665,7 @@
         <v>34</v>
       </c>
       <c r="E376" t="s">
-        <v>729</v>
+        <v>733</v>
       </c>
       <c r="F376" t="s">
         <v>40</v>
@@ -23739,7 +23739,7 @@
         <v>530</v>
       </c>
       <c r="K377" t="s">
-        <v>727</v>
+        <v>728</v>
       </c>
       <c r="L377" t="s">
         <v>34</v>
@@ -23795,7 +23795,7 @@
         <v>179</v>
       </c>
       <c r="K378" t="s">
-        <v>727</v>
+        <v>728</v>
       </c>
       <c r="L378" t="s">
         <v>34</v>
@@ -23833,7 +23833,7 @@
         <v>34</v>
       </c>
       <c r="E379" t="s">
-        <v>720</v>
+        <v>724</v>
       </c>
       <c r="F379" t="s">
         <v>40</v>
@@ -23848,7 +23848,7 @@
         <v>772</v>
       </c>
       <c r="J379" t="s">
-        <v>726</v>
+        <v>727</v>
       </c>
       <c r="K379" t="s">
         <v>45</v>
@@ -23889,7 +23889,7 @@
         <v>34</v>
       </c>
       <c r="E380" t="s">
-        <v>720</v>
+        <v>724</v>
       </c>
       <c r="F380" t="s">
         <v>40</v>
@@ -23904,7 +23904,7 @@
         <v>750</v>
       </c>
       <c r="J380" t="s">
-        <v>726</v>
+        <v>727</v>
       </c>
       <c r="K380" t="s">
         <v>45</v>
@@ -23945,7 +23945,7 @@
         <v>34</v>
       </c>
       <c r="E381" t="s">
-        <v>720</v>
+        <v>724</v>
       </c>
       <c r="F381" t="s">
         <v>40</v>
@@ -24001,7 +24001,7 @@
         <v>34</v>
       </c>
       <c r="E382" t="s">
-        <v>720</v>
+        <v>724</v>
       </c>
       <c r="F382" t="s">
         <v>40</v>
@@ -24016,7 +24016,7 @@
         <v>780</v>
       </c>
       <c r="J382" t="s">
-        <v>726</v>
+        <v>727</v>
       </c>
       <c r="K382" t="s">
         <v>45</v>
@@ -24113,7 +24113,7 @@
         <v>34</v>
       </c>
       <c r="E384" t="s">
-        <v>720</v>
+        <v>724</v>
       </c>
       <c r="F384" t="s">
         <v>40</v>
@@ -24128,7 +24128,7 @@
         <v>785</v>
       </c>
       <c r="J384" t="s">
-        <v>726</v>
+        <v>727</v>
       </c>
       <c r="K384" t="s">
         <v>45</v>
@@ -24281,7 +24281,7 @@
         <v>34</v>
       </c>
       <c r="E387" t="s">
-        <v>720</v>
+        <v>724</v>
       </c>
       <c r="F387" t="s">
         <v>40</v>
@@ -24296,7 +24296,7 @@
         <v>791</v>
       </c>
       <c r="J387" t="s">
-        <v>726</v>
+        <v>727</v>
       </c>
       <c r="K387" t="s">
         <v>45</v>
@@ -24738,7 +24738,7 @@
         <v>41</v>
       </c>
       <c r="H395" t="s">
-        <v>197</v>
+        <v>192</v>
       </c>
       <c r="I395" t="s">
         <v>810</v>
@@ -24968,7 +24968,7 @@
         <v>819</v>
       </c>
       <c r="J399" t="s">
-        <v>736</v>
+        <v>722</v>
       </c>
       <c r="K399" t="s">
         <v>68</v>
@@ -25136,10 +25136,10 @@
         <v>828</v>
       </c>
       <c r="J402" t="s">
-        <v>726</v>
+        <v>727</v>
       </c>
       <c r="K402" t="s">
-        <v>727</v>
+        <v>728</v>
       </c>
       <c r="L402" t="s">
         <v>829</v>
@@ -25401,7 +25401,7 @@
         <v>33</v>
       </c>
       <c r="E407" t="s">
-        <v>720</v>
+        <v>724</v>
       </c>
       <c r="F407" t="s">
         <v>40</v>
@@ -25416,7 +25416,7 @@
         <v>848</v>
       </c>
       <c r="J407" t="s">
-        <v>726</v>
+        <v>727</v>
       </c>
       <c r="K407" t="s">
         <v>45</v>
@@ -25569,7 +25569,7 @@
         <v>33</v>
       </c>
       <c r="E410" t="s">
-        <v>720</v>
+        <v>724</v>
       </c>
       <c r="F410" t="s">
         <v>40</v>
@@ -25584,7 +25584,7 @@
         <v>860</v>
       </c>
       <c r="J410" t="s">
-        <v>726</v>
+        <v>727</v>
       </c>
       <c r="K410" t="s">
         <v>320</v>
@@ -25696,10 +25696,10 @@
         <v>866</v>
       </c>
       <c r="J412" t="s">
-        <v>726</v>
+        <v>727</v>
       </c>
       <c r="K412" t="s">
-        <v>727</v>
+        <v>728</v>
       </c>
       <c r="L412" t="s">
         <v>867</v>
@@ -25811,10 +25811,10 @@
         <v>179</v>
       </c>
       <c r="K414" t="s">
-        <v>293</v>
+        <v>664</v>
       </c>
       <c r="L414" t="s">
-        <v>34</v>
+        <v>874</v>
       </c>
       <c r="M414" t="s">
         <v>870</v>
@@ -25849,7 +25849,7 @@
         <v>34</v>
       </c>
       <c r="E415" t="s">
-        <v>874</v>
+        <v>875</v>
       </c>
       <c r="F415" t="s">
         <v>208</v>
@@ -25858,16 +25858,16 @@
         <v>41</v>
       </c>
       <c r="H415" t="s">
-        <v>875</v>
+        <v>876</v>
       </c>
       <c r="I415" t="s">
-        <v>876</v>
+        <v>877</v>
       </c>
       <c r="J415" t="s">
         <v>179</v>
       </c>
       <c r="K415" t="s">
-        <v>109</v>
+        <v>293</v>
       </c>
       <c r="L415" t="s">
         <v>34</v>
@@ -25882,7 +25882,7 @@
         <v>48</v>
       </c>
       <c r="P415" t="s">
-        <v>876</v>
+        <v>877</v>
       </c>
       <c r="Q415" t="s">
         <v>47</v>
@@ -25905,7 +25905,7 @@
         <v>34</v>
       </c>
       <c r="E416" t="s">
-        <v>877</v>
+        <v>878</v>
       </c>
       <c r="F416" t="s">
         <v>208</v>
@@ -25914,19 +25914,19 @@
         <v>41</v>
       </c>
       <c r="H416" t="s">
-        <v>878</v>
+        <v>879</v>
       </c>
       <c r="I416" t="s">
-        <v>879</v>
+        <v>880</v>
       </c>
       <c r="J416" t="s">
         <v>179</v>
       </c>
       <c r="K416" t="s">
-        <v>664</v>
+        <v>109</v>
       </c>
       <c r="L416" t="s">
-        <v>880</v>
+        <v>34</v>
       </c>
       <c r="M416" t="s">
         <v>870</v>
@@ -25938,7 +25938,7 @@
         <v>48</v>
       </c>
       <c r="P416" t="s">
-        <v>879</v>
+        <v>880</v>
       </c>
       <c r="Q416" t="s">
         <v>47</v>
@@ -26129,7 +26129,7 @@
         <v>33</v>
       </c>
       <c r="E420" t="s">
-        <v>720</v>
+        <v>724</v>
       </c>
       <c r="F420" t="s">
         <v>40</v>
@@ -26144,7 +26144,7 @@
         <v>893</v>
       </c>
       <c r="J420" t="s">
-        <v>726</v>
+        <v>727</v>
       </c>
       <c r="K420" t="s">
         <v>45</v>
@@ -26356,25 +26356,25 @@
         <v>908</v>
       </c>
       <c r="F424" t="s">
-        <v>208</v>
+        <v>40</v>
       </c>
       <c r="G424" t="s">
         <v>41</v>
       </c>
       <c r="H424" t="s">
+        <v>903</v>
+      </c>
+      <c r="I424" t="s">
         <v>909</v>
       </c>
-      <c r="I424" t="s">
+      <c r="J424" t="s">
+        <v>373</v>
+      </c>
+      <c r="K424" t="s">
+        <v>45</v>
+      </c>
+      <c r="L424" t="s">
         <v>910</v>
-      </c>
-      <c r="J424" t="s">
-        <v>179</v>
-      </c>
-      <c r="K424" t="s">
-        <v>293</v>
-      </c>
-      <c r="L424" t="s">
-        <v>34</v>
       </c>
       <c r="M424" t="s">
         <v>907</v>
@@ -26386,7 +26386,7 @@
         <v>48</v>
       </c>
       <c r="P424" t="s">
-        <v>910</v>
+        <v>909</v>
       </c>
       <c r="Q424" t="s">
         <v>47</v>
@@ -26409,7 +26409,7 @@
         <v>34</v>
       </c>
       <c r="E425" t="s">
-        <v>720</v>
+        <v>724</v>
       </c>
       <c r="F425" t="s">
         <v>40</v>
@@ -26418,19 +26418,19 @@
         <v>41</v>
       </c>
       <c r="H425" t="s">
+        <v>903</v>
+      </c>
+      <c r="I425" t="s">
         <v>911</v>
-      </c>
-      <c r="I425" t="s">
-        <v>912</v>
       </c>
       <c r="J425" t="s">
         <v>369</v>
       </c>
       <c r="K425" t="s">
-        <v>45</v>
+        <v>674</v>
       </c>
       <c r="L425" t="s">
-        <v>913</v>
+        <v>912</v>
       </c>
       <c r="M425" t="s">
         <v>907</v>
@@ -26442,7 +26442,7 @@
         <v>48</v>
       </c>
       <c r="P425" t="s">
-        <v>912</v>
+        <v>911</v>
       </c>
       <c r="Q425" t="s">
         <v>47</v>
@@ -26465,28 +26465,28 @@
         <v>34</v>
       </c>
       <c r="E426" t="s">
-        <v>720</v>
+        <v>913</v>
       </c>
       <c r="F426" t="s">
-        <v>40</v>
+        <v>208</v>
       </c>
       <c r="G426" t="s">
         <v>41</v>
       </c>
       <c r="H426" t="s">
-        <v>903</v>
+        <v>914</v>
       </c>
       <c r="I426" t="s">
-        <v>914</v>
+        <v>915</v>
       </c>
       <c r="J426" t="s">
-        <v>369</v>
+        <v>179</v>
       </c>
       <c r="K426" t="s">
-        <v>674</v>
+        <v>293</v>
       </c>
       <c r="L426" t="s">
-        <v>915</v>
+        <v>34</v>
       </c>
       <c r="M426" t="s">
         <v>907</v>
@@ -26498,7 +26498,7 @@
         <v>48</v>
       </c>
       <c r="P426" t="s">
-        <v>914</v>
+        <v>915</v>
       </c>
       <c r="Q426" t="s">
         <v>47</v>
@@ -26521,7 +26521,7 @@
         <v>34</v>
       </c>
       <c r="E427" t="s">
-        <v>916</v>
+        <v>724</v>
       </c>
       <c r="F427" t="s">
         <v>40</v>
@@ -26530,13 +26530,13 @@
         <v>41</v>
       </c>
       <c r="H427" t="s">
-        <v>903</v>
+        <v>916</v>
       </c>
       <c r="I427" t="s">
         <v>917</v>
       </c>
       <c r="J427" t="s">
-        <v>373</v>
+        <v>369</v>
       </c>
       <c r="K427" t="s">
         <v>45</v>
@@ -26745,7 +26745,7 @@
         <v>33</v>
       </c>
       <c r="E431" t="s">
-        <v>720</v>
+        <v>724</v>
       </c>
       <c r="F431" t="s">
         <v>40</v>
@@ -26760,7 +26760,7 @@
         <v>930</v>
       </c>
       <c r="J431" t="s">
-        <v>726</v>
+        <v>727</v>
       </c>
       <c r="K431" t="s">
         <v>45</v>
@@ -26913,7 +26913,7 @@
         <v>33</v>
       </c>
       <c r="E434" t="s">
-        <v>826</v>
+        <v>724</v>
       </c>
       <c r="F434" t="s">
         <v>40</v>
@@ -26928,10 +26928,10 @@
         <v>942</v>
       </c>
       <c r="J434" t="s">
-        <v>736</v>
+        <v>727</v>
       </c>
       <c r="K434" t="s">
-        <v>67</v>
+        <v>45</v>
       </c>
       <c r="L434" t="s">
         <v>943</v>
@@ -26969,7 +26969,7 @@
         <v>34</v>
       </c>
       <c r="E435" t="s">
-        <v>720</v>
+        <v>826</v>
       </c>
       <c r="F435" t="s">
         <v>40</v>
@@ -26984,10 +26984,10 @@
         <v>945</v>
       </c>
       <c r="J435" t="s">
-        <v>726</v>
+        <v>722</v>
       </c>
       <c r="K435" t="s">
-        <v>45</v>
+        <v>67</v>
       </c>
       <c r="L435" t="s">
         <v>946</v>
@@ -27193,7 +27193,7 @@
         <v>33</v>
       </c>
       <c r="E439" t="s">
-        <v>729</v>
+        <v>733</v>
       </c>
       <c r="F439" t="s">
         <v>40</v>
@@ -28119,7 +28119,7 @@
         <v>47</v>
       </c>
       <c r="O455" t="s">
-        <v>412</v>
+        <v>385</v>
       </c>
       <c r="P455" t="s">
         <v>975</v>

</xml_diff>